<commit_message>
sync(workvault): 2026-10-26 18:22 差分 3 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/LNB管理手順書案_未承認.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/LNB管理手順書案_未承認.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nk365-my.sharepoint.com/personal/ss80751_ad_nkc_co_jp/Documents/ドキュメント/Work_Vault/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="6_{C0F3EAFA-DEEC-4CD0-B5EF-21988F4F198C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3754AFE-D5C1-4732-9B70-9CD38C154FAE}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="6_{C0F3EAFA-DEEC-4CD0-B5EF-21988F4F198C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E526E21C-A2AF-49D8-835E-6CDF4B701051}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2238,79 +2238,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2352,6 +2279,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="3" applyFont="1" applyBorder="1"/>
@@ -2362,6 +2298,70 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -6762,7 +6762,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="50800" tIns="25400" rIns="25400" bIns="12700" rtlCol="0" anchor="t"/>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="50800" tIns="25400" rIns="76200" bIns="12700" rtlCol="0" anchor="t" anchorCtr="1"/>
         <a:lstStyle/>
         <a:p>
           <a:pPr algn="l"/>
@@ -8792,23 +8792,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>27940</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>93980</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>123190</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>73660</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>27940</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>123190</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>40640</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="20" name="rel_e1">
+        <xdr:cNvPr id="36" name="rel_e1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0F5867DD-F96E-5C6A-8CF2-53A830ADD8A9}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CB902B3-CE31-D570-65AF-B918F91388C9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8816,7 +8816,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2489200" y="4292600"/>
+          <a:off x="1936750" y="2832100"/>
           <a:ext cx="0" cy="927100"/>
         </a:xfrm>
         <a:prstGeom prst="line">
@@ -8848,23 +8848,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>104140</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>104140</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>96520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
-      <xdr:colOff>88900</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>83820</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>48260</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="rel_l_e1">
+        <xdr:cNvPr id="37" name="rel_l_e1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF62F59A-123F-5351-7DA6-80B077677102}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEE59891-6159-3494-E572-15BB290B6E2D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8872,7 +8872,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2565400" y="4622800"/>
+          <a:off x="2006600" y="3175000"/>
           <a:ext cx="762000" cy="139700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -8917,7 +8917,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="25400" tIns="12700" rIns="25400" bIns="12700" rtlCol="0" anchor="ctr" anchorCtr="0">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
@@ -8939,23 +8939,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>43180</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>2540</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>81280</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>58420</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>2540</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>17780</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>66040</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="22" name="rel_e2">
+        <xdr:cNvPr id="38" name="rel_e2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC75B970-A3E0-3063-7A5D-5407D1CDADF4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3973E9B2-51A1-9F86-36F8-438BDF8CE773}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8963,8 +8963,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="3670300" y="4140200"/>
-          <a:ext cx="533400" cy="1181100"/>
+          <a:off x="3111500" y="2679700"/>
+          <a:ext cx="533400" cy="1104900"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -8995,23 +8995,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>55880</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>73660</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>99060</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>96520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>45720</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>53340</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>88900</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="23" name="rel_l_e2">
+        <xdr:cNvPr id="39" name="rel_l_e2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DF8BC6D-02BB-CD30-F9F6-7557D5A2B6FF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD823484-D694-5ECC-A4FD-ED88E05B5393}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9019,7 +9019,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3683000" y="4432300"/>
+          <a:off x="2819400" y="3175000"/>
           <a:ext cx="508000" cy="139700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9064,7 +9064,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="25400" tIns="12700" rIns="25400" bIns="12700" rtlCol="0" anchor="ctr" anchorCtr="0">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
@@ -9086,23 +9086,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>43180</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>2540</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>58420</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>2540</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>17780</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>142240</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="24" name="rel_e3">
+        <xdr:cNvPr id="40" name="rel_e3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3C43119-CB08-F98F-EC85-1FFBC9DA4011}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{274975B1-0E48-E324-B090-87A5FBA227CA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9110,8 +9110,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3670300" y="5778500"/>
-          <a:ext cx="533400" cy="1943100"/>
+          <a:off x="3111500" y="4343400"/>
+          <a:ext cx="533400" cy="1917700"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -9142,23 +9142,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>68580</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>33020</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>78740</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>25400</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>12700</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>35560</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="rel_l_e3">
+        <xdr:cNvPr id="41" name="rel_l_e3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F916300-2DA5-ACF5-6410-B710476427F2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F4F5E936-0A98-202B-3CFA-7C74A6C5CC0F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9166,7 +9166,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3048000" y="7112000"/>
+          <a:off x="2540000" y="5651500"/>
           <a:ext cx="863600" cy="139700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9211,7 +9211,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="25400" tIns="12700" rIns="25400" bIns="12700" rtlCol="0" anchor="ctr" anchorCtr="0">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
@@ -9253,23 +9253,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>104140</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>10160</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>149860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>50800</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>60960</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>17780</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="26" name="rel_e4">
+        <xdr:cNvPr id="42" name="rel_e4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5B815E7-C484-862E-70BF-6252CE34AE4E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5322D314-BC07-A055-5FC7-59033052FB74}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9277,8 +9277,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="1917700" y="6769100"/>
-          <a:ext cx="76200" cy="2108200"/>
+          <a:off x="1358900" y="5308600"/>
+          <a:ext cx="127000" cy="2108200"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -9309,23 +9309,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>48260</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5080</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>116840</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>86360</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="rel_l_e4">
+        <xdr:cNvPr id="43" name="rel_l_e4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F73A8509-41CB-F95E-428D-0EDFC068B1E7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6FB8D9A-42A5-CCFA-5362-0480AB06A45E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9333,7 +9333,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1473200" y="8204200"/>
+          <a:off x="914400" y="6705600"/>
           <a:ext cx="457200" cy="139700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9378,7 +9378,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="25400" tIns="12700" rIns="25400" bIns="12700" rtlCol="0" anchor="ctr" anchorCtr="0">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
@@ -9410,23 +9410,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>5080</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>10160</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>149860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>48260</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>17780</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="28" name="rel_e5">
+        <xdr:cNvPr id="44" name="rel_e5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5B3F3AD8-974E-9DB9-4647-0B0B2DFC1388}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D82E7207-684D-E838-40DD-0C393C30028E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9434,8 +9434,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1" flipV="1">
-          <a:off x="2984500" y="6769100"/>
-          <a:ext cx="431800" cy="2108200"/>
+          <a:off x="2476500" y="5308600"/>
+          <a:ext cx="381000" cy="2108200"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -9466,23 +9466,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>58420</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>5080</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>78740</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>144780</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>88900</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>124460</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="rel_l_e5">
+        <xdr:cNvPr id="45" name="rel_l_e5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F67FD1AA-6A67-2F8C-CD71-6B0A40CC6619}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C0C89AF-6E04-0611-D314-EF8A3C47E5BB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9490,7 +9490,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3556000" y="8204200"/>
+          <a:off x="3048000" y="6743700"/>
           <a:ext cx="279400" cy="139700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9535,7 +9535,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="25400" tIns="12700" rIns="25400" bIns="12700" rtlCol="0" anchor="ctr" anchorCtr="0">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
@@ -9557,23 +9557,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>43180</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>2540</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>96520</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>55880</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>119380</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="30" name="rel_e6">
+        <xdr:cNvPr id="46" name="rel_e6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E65F93EB-BC7D-97C6-A17C-335FF3DC9721}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9151CDC2-4ABD-6471-7674-44F05935918A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9581,8 +9581,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1" flipV="1">
-          <a:off x="3670300" y="5702300"/>
-          <a:ext cx="1219200" cy="76200"/>
+          <a:off x="3111500" y="4191000"/>
+          <a:ext cx="1219200" cy="127000"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -9613,23 +9613,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>43180</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>83820</xdr:rowOff>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>104140</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>5080</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="31" name="rel_l_e6">
+        <xdr:cNvPr id="47" name="rel_l_e6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A7877C5-0CBE-3B6C-87BA-816F5D086462}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{59A74420-F9F2-2AA1-AB63-99252C52D99C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9637,7 +9637,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4318000" y="5562600"/>
+          <a:off x="4597400" y="4064000"/>
           <a:ext cx="558800" cy="139700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9682,7 +9682,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="25400" tIns="12700" rIns="25400" bIns="12700" rtlCol="0" anchor="ctr" anchorCtr="0">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
@@ -9704,23 +9704,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>43180</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>83820</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>2540</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>49</xdr:col>
-      <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
+      <xdr:col>44</xdr:col>
+      <xdr:colOff>91440</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>119380</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="32" name="rel_e7">
+        <xdr:cNvPr id="48" name="rel_e7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8827E2BD-7F86-99F0-390D-AF9B69E51E02}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E554EA2-9AD2-0D54-677C-79078377B600}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9728,8 +9728,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1" flipV="1">
-          <a:off x="3670300" y="5562600"/>
-          <a:ext cx="2679700" cy="215900"/>
+          <a:off x="3111500" y="4038600"/>
+          <a:ext cx="2679700" cy="279400"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -9761,22 +9761,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>40</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>20320</xdr:rowOff>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>42</xdr:col>
-      <xdr:colOff>20320</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>81280</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="33" name="rel_l_e7">
+        <xdr:cNvPr id="49" name="rel_l_e7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{49BDD18E-DDE0-34B7-486C-17C4BA693EAF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5A1C0D13-AF15-05FF-924B-52C874D424D4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9784,7 +9784,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5181600" y="5499100"/>
+          <a:off x="5207000" y="4140200"/>
           <a:ext cx="279400" cy="139700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9829,7 +9829,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="25400" tIns="12700" rIns="25400" bIns="12700" rtlCol="0" anchor="ctr" anchorCtr="0">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
@@ -9851,23 +9851,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>43180</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>10160</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>2540</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>149860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>42</xdr:col>
-      <xdr:colOff>109220</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>104140</xdr:rowOff>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>74930</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="34" name="rel_e8">
+        <xdr:cNvPr id="50" name="rel_e8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{61B5E362-71B5-C02C-7490-ED1B358CC785}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1935CA14-9E28-C237-B48F-75D7DD470DB7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9875,8 +9875,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="3670300" y="5168900"/>
-          <a:ext cx="1879600" cy="254000"/>
+          <a:off x="3111500" y="3708400"/>
+          <a:ext cx="1885950" cy="177800"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -9907,23 +9907,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>63500</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>73660</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>154940</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>44</xdr:col>
-      <xdr:colOff>66040</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>154940</xdr:rowOff>
+      <xdr:col>40</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>134620</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="35" name="rel_l_e8">
+        <xdr:cNvPr id="51" name="rel_l_e8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B66EC1CB-957A-6F7F-58EE-2345EB7B1C16}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EFE557A9-829F-F5A0-C9B4-046603CE8A53}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -9931,7 +9931,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4597400" y="5334000"/>
+          <a:off x="4089400" y="3873500"/>
           <a:ext cx="1168400" cy="139700"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -9976,7 +9976,7 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="25400" tIns="12700" rIns="25400" bIns="12700" rtlCol="0" anchor="ctr" anchorCtr="0">
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr" anchorCtr="0">
           <a:noAutofit/>
         </a:bodyPr>
         <a:lstStyle/>
@@ -10970,102 +10970,102 @@
       </c>
       <c r="N1" s="25"/>
       <c r="O1" s="26"/>
-      <c r="P1" s="76"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="77"/>
-      <c r="T1" s="77"/>
-      <c r="U1" s="77"/>
-      <c r="V1" s="78"/>
+      <c r="P1" s="104"/>
+      <c r="Q1" s="105"/>
+      <c r="R1" s="105"/>
+      <c r="S1" s="105"/>
+      <c r="T1" s="105"/>
+      <c r="U1" s="105"/>
+      <c r="V1" s="106"/>
       <c r="W1" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="79" t="s">
+      <c r="X1" s="99" t="s">
         <v>347</v>
       </c>
-      <c r="Y1" s="80"/>
+      <c r="Y1" s="100"/>
     </row>
     <row r="2" spans="1:25" ht="58.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="29"/>
       <c r="B2" s="30"/>
-      <c r="D2" s="81" t="s">
+      <c r="D2" s="101" t="s">
         <v>348</v>
       </c>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82"/>
-      <c r="K2" s="82"/>
-      <c r="L2" s="82"/>
-      <c r="M2" s="82"/>
-      <c r="N2" s="82"/>
-      <c r="O2" s="82"/>
-      <c r="P2" s="82"/>
-      <c r="Q2" s="82"/>
-      <c r="R2" s="82"/>
-      <c r="S2" s="82"/>
-      <c r="T2" s="82"/>
-      <c r="U2" s="82"/>
-      <c r="V2" s="82"/>
-      <c r="W2" s="82"/>
+      <c r="E2" s="102"/>
+      <c r="F2" s="102"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="102"/>
+      <c r="I2" s="102"/>
+      <c r="J2" s="102"/>
+      <c r="K2" s="102"/>
+      <c r="L2" s="102"/>
+      <c r="M2" s="102"/>
+      <c r="N2" s="102"/>
+      <c r="O2" s="102"/>
+      <c r="P2" s="102"/>
+      <c r="Q2" s="102"/>
+      <c r="R2" s="102"/>
+      <c r="S2" s="102"/>
+      <c r="T2" s="102"/>
+      <c r="U2" s="102"/>
+      <c r="V2" s="102"/>
+      <c r="W2" s="102"/>
       <c r="X2" s="31"/>
       <c r="Y2" s="23"/>
     </row>
     <row r="3" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="32"/>
       <c r="B3" s="33"/>
-      <c r="D3" s="83" t="s">
+      <c r="D3" s="103" t="s">
         <v>349</v>
       </c>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
-      <c r="J3" s="83"/>
-      <c r="K3" s="83"/>
-      <c r="L3" s="83"/>
-      <c r="M3" s="83"/>
-      <c r="N3" s="83"/>
-      <c r="O3" s="83"/>
-      <c r="P3" s="83"/>
-      <c r="Q3" s="83"/>
-      <c r="R3" s="83"/>
-      <c r="S3" s="83"/>
-      <c r="T3" s="83"/>
-      <c r="U3" s="83"/>
-      <c r="V3" s="83"/>
-      <c r="W3" s="83"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="103"/>
+      <c r="I3" s="103"/>
+      <c r="J3" s="103"/>
+      <c r="K3" s="103"/>
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
+      <c r="N3" s="103"/>
+      <c r="O3" s="103"/>
+      <c r="P3" s="103"/>
+      <c r="Q3" s="103"/>
+      <c r="R3" s="103"/>
+      <c r="S3" s="103"/>
+      <c r="T3" s="103"/>
+      <c r="U3" s="103"/>
+      <c r="V3" s="103"/>
+      <c r="W3" s="103"/>
       <c r="X3" s="33"/>
       <c r="Y3" s="34"/>
     </row>
     <row r="4" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="32"/>
       <c r="B4" s="33"/>
-      <c r="D4" s="83" t="s">
+      <c r="D4" s="103" t="s">
         <v>350</v>
       </c>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
-      <c r="H4" s="83"/>
-      <c r="I4" s="83"/>
-      <c r="J4" s="83"/>
-      <c r="K4" s="83"/>
-      <c r="L4" s="83"/>
-      <c r="M4" s="83"/>
-      <c r="N4" s="83"/>
-      <c r="O4" s="83"/>
-      <c r="P4" s="83"/>
-      <c r="Q4" s="83"/>
-      <c r="R4" s="83"/>
-      <c r="S4" s="83"/>
-      <c r="T4" s="83"/>
-      <c r="U4" s="83"/>
-      <c r="V4" s="83"/>
-      <c r="W4" s="83"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="103"/>
+      <c r="G4" s="103"/>
+      <c r="H4" s="103"/>
+      <c r="I4" s="103"/>
+      <c r="J4" s="103"/>
+      <c r="K4" s="103"/>
+      <c r="L4" s="103"/>
+      <c r="M4" s="103"/>
+      <c r="N4" s="103"/>
+      <c r="O4" s="103"/>
+      <c r="P4" s="103"/>
+      <c r="Q4" s="103"/>
+      <c r="R4" s="103"/>
+      <c r="S4" s="103"/>
+      <c r="T4" s="103"/>
+      <c r="U4" s="103"/>
+      <c r="V4" s="103"/>
+      <c r="W4" s="103"/>
       <c r="X4" s="33"/>
       <c r="Y4" s="34"/>
     </row>
@@ -11109,21 +11109,21 @@
       <c r="K6" s="33"/>
       <c r="L6" s="36"/>
       <c r="M6" s="36"/>
-      <c r="O6" s="76" t="s">
+      <c r="O6" s="104" t="s">
         <v>351</v>
       </c>
-      <c r="P6" s="77"/>
-      <c r="Q6" s="78"/>
-      <c r="R6" s="76" t="s">
+      <c r="P6" s="105"/>
+      <c r="Q6" s="106"/>
+      <c r="R6" s="104" t="s">
         <v>352</v>
       </c>
-      <c r="S6" s="77"/>
-      <c r="T6" s="78"/>
-      <c r="U6" s="76" t="s">
+      <c r="S6" s="105"/>
+      <c r="T6" s="106"/>
+      <c r="U6" s="104" t="s">
         <v>353</v>
       </c>
-      <c r="V6" s="77"/>
-      <c r="W6" s="78"/>
+      <c r="V6" s="105"/>
+      <c r="W6" s="106"/>
       <c r="Y6" s="34"/>
     </row>
     <row r="7" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -11140,15 +11140,15 @@
       <c r="K7" s="33"/>
       <c r="L7" s="36"/>
       <c r="M7" s="36"/>
-      <c r="O7" s="67"/>
-      <c r="P7" s="68"/>
-      <c r="Q7" s="69"/>
-      <c r="R7" s="67"/>
-      <c r="S7" s="68"/>
-      <c r="T7" s="69"/>
-      <c r="U7" s="67"/>
-      <c r="V7" s="68"/>
-      <c r="W7" s="69"/>
+      <c r="O7" s="107"/>
+      <c r="P7" s="108"/>
+      <c r="Q7" s="109"/>
+      <c r="R7" s="107"/>
+      <c r="S7" s="108"/>
+      <c r="T7" s="109"/>
+      <c r="U7" s="107"/>
+      <c r="V7" s="108"/>
+      <c r="W7" s="109"/>
       <c r="Y7" s="34"/>
     </row>
     <row r="8" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11165,15 +11165,15 @@
       <c r="K8" s="33"/>
       <c r="L8" s="36"/>
       <c r="M8" s="36"/>
-      <c r="O8" s="70"/>
-      <c r="P8" s="71"/>
-      <c r="Q8" s="72"/>
-      <c r="R8" s="70"/>
-      <c r="S8" s="71"/>
-      <c r="T8" s="72"/>
-      <c r="U8" s="70"/>
-      <c r="V8" s="71"/>
-      <c r="W8" s="72"/>
+      <c r="O8" s="110"/>
+      <c r="P8" s="111"/>
+      <c r="Q8" s="112"/>
+      <c r="R8" s="110"/>
+      <c r="S8" s="111"/>
+      <c r="T8" s="112"/>
+      <c r="U8" s="110"/>
+      <c r="V8" s="111"/>
+      <c r="W8" s="112"/>
       <c r="Y8" s="34"/>
     </row>
     <row r="9" spans="1:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -11217,18 +11217,18 @@
       <c r="L10" s="36"/>
       <c r="M10" s="36"/>
       <c r="N10" s="36"/>
-      <c r="P10" s="73" t="s">
+      <c r="P10" s="113" t="s">
         <v>354</v>
       </c>
-      <c r="Q10" s="73"/>
-      <c r="R10" s="73"/>
-      <c r="S10" s="74" t="s">
+      <c r="Q10" s="113"/>
+      <c r="R10" s="113"/>
+      <c r="S10" s="114" t="s">
         <v>355</v>
       </c>
-      <c r="T10" s="74"/>
-      <c r="U10" s="74"/>
-      <c r="V10" s="74"/>
-      <c r="W10" s="74"/>
+      <c r="T10" s="114"/>
+      <c r="U10" s="114"/>
+      <c r="V10" s="114"/>
+      <c r="W10" s="114"/>
       <c r="Y10" s="34"/>
     </row>
     <row r="11" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -11246,27 +11246,27 @@
       <c r="L11" s="36"/>
       <c r="M11" s="36"/>
       <c r="N11" s="36"/>
-      <c r="P11" s="66" t="s">
+      <c r="P11" s="97" t="s">
         <v>356</v>
       </c>
-      <c r="Q11" s="66"/>
-      <c r="R11" s="66"/>
-      <c r="S11" s="75" t="s">
+      <c r="Q11" s="97"/>
+      <c r="R11" s="97"/>
+      <c r="S11" s="115" t="s">
         <v>355</v>
       </c>
-      <c r="T11" s="75"/>
-      <c r="U11" s="75"/>
-      <c r="V11" s="75"/>
-      <c r="W11" s="75"/>
+      <c r="T11" s="115"/>
+      <c r="U11" s="115"/>
+      <c r="V11" s="115"/>
+      <c r="W11" s="115"/>
       <c r="Y11" s="34"/>
     </row>
     <row r="12" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="37"/>
-      <c r="P12" s="66" t="s">
+      <c r="P12" s="97" t="s">
         <v>357</v>
       </c>
-      <c r="Q12" s="66"/>
-      <c r="R12" s="66"/>
+      <c r="Q12" s="97"/>
+      <c r="R12" s="97"/>
       <c r="S12" s="38"/>
       <c r="T12" s="38"/>
       <c r="U12" s="39" t="s">
@@ -11288,642 +11288,642 @@
         <v>360</v>
       </c>
       <c r="B14" s="44"/>
-      <c r="C14" s="84"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="66"/>
-      <c r="F14" s="85"/>
-      <c r="G14" s="84"/>
-      <c r="H14" s="66"/>
-      <c r="I14" s="66"/>
-      <c r="J14" s="85"/>
-      <c r="K14" s="86"/>
-      <c r="L14" s="87"/>
-      <c r="M14" s="87"/>
-      <c r="N14" s="87"/>
-      <c r="O14" s="87"/>
-      <c r="P14" s="87"/>
-      <c r="Q14" s="88"/>
-      <c r="R14" s="84"/>
-      <c r="S14" s="85"/>
-      <c r="T14" s="84"/>
-      <c r="U14" s="66"/>
-      <c r="V14" s="66"/>
-      <c r="W14" s="85"/>
-      <c r="X14" s="84"/>
-      <c r="Y14" s="85"/>
+      <c r="C14" s="95"/>
+      <c r="D14" s="97"/>
+      <c r="E14" s="97"/>
+      <c r="F14" s="96"/>
+      <c r="G14" s="95"/>
+      <c r="H14" s="97"/>
+      <c r="I14" s="97"/>
+      <c r="J14" s="96"/>
+      <c r="K14" s="98"/>
+      <c r="L14" s="93"/>
+      <c r="M14" s="93"/>
+      <c r="N14" s="93"/>
+      <c r="O14" s="93"/>
+      <c r="P14" s="93"/>
+      <c r="Q14" s="94"/>
+      <c r="R14" s="95"/>
+      <c r="S14" s="96"/>
+      <c r="T14" s="95"/>
+      <c r="U14" s="97"/>
+      <c r="V14" s="97"/>
+      <c r="W14" s="96"/>
+      <c r="X14" s="95"/>
+      <c r="Y14" s="96"/>
     </row>
     <row r="15" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B15" s="44"/>
-      <c r="C15" s="84"/>
-      <c r="D15" s="66"/>
-      <c r="E15" s="66"/>
-      <c r="F15" s="85"/>
-      <c r="G15" s="84"/>
-      <c r="H15" s="66"/>
-      <c r="I15" s="66"/>
-      <c r="J15" s="85"/>
-      <c r="K15" s="86"/>
-      <c r="L15" s="87"/>
-      <c r="M15" s="87"/>
-      <c r="N15" s="87"/>
-      <c r="O15" s="87"/>
-      <c r="P15" s="87"/>
-      <c r="Q15" s="88"/>
-      <c r="R15" s="84"/>
-      <c r="S15" s="85"/>
-      <c r="T15" s="84"/>
-      <c r="U15" s="66"/>
-      <c r="V15" s="66"/>
-      <c r="W15" s="85"/>
-      <c r="X15" s="84"/>
-      <c r="Y15" s="85"/>
+      <c r="C15" s="95"/>
+      <c r="D15" s="97"/>
+      <c r="E15" s="97"/>
+      <c r="F15" s="96"/>
+      <c r="G15" s="95"/>
+      <c r="H15" s="97"/>
+      <c r="I15" s="97"/>
+      <c r="J15" s="96"/>
+      <c r="K15" s="98"/>
+      <c r="L15" s="93"/>
+      <c r="M15" s="93"/>
+      <c r="N15" s="93"/>
+      <c r="O15" s="93"/>
+      <c r="P15" s="93"/>
+      <c r="Q15" s="94"/>
+      <c r="R15" s="95"/>
+      <c r="S15" s="96"/>
+      <c r="T15" s="95"/>
+      <c r="U15" s="97"/>
+      <c r="V15" s="97"/>
+      <c r="W15" s="96"/>
+      <c r="X15" s="95"/>
+      <c r="Y15" s="96"/>
     </row>
     <row r="16" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B16" s="44"/>
-      <c r="C16" s="84"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="66"/>
-      <c r="F16" s="85"/>
-      <c r="G16" s="84"/>
-      <c r="H16" s="66"/>
-      <c r="I16" s="66"/>
-      <c r="J16" s="85"/>
-      <c r="K16" s="86"/>
-      <c r="L16" s="87"/>
-      <c r="M16" s="87"/>
-      <c r="N16" s="87"/>
-      <c r="O16" s="87"/>
-      <c r="P16" s="87"/>
-      <c r="Q16" s="88"/>
-      <c r="R16" s="84"/>
-      <c r="S16" s="85"/>
-      <c r="T16" s="84"/>
-      <c r="U16" s="66"/>
-      <c r="V16" s="66"/>
-      <c r="W16" s="85"/>
-      <c r="X16" s="84"/>
-      <c r="Y16" s="85"/>
+      <c r="C16" s="95"/>
+      <c r="D16" s="97"/>
+      <c r="E16" s="97"/>
+      <c r="F16" s="96"/>
+      <c r="G16" s="95"/>
+      <c r="H16" s="97"/>
+      <c r="I16" s="97"/>
+      <c r="J16" s="96"/>
+      <c r="K16" s="98"/>
+      <c r="L16" s="93"/>
+      <c r="M16" s="93"/>
+      <c r="N16" s="93"/>
+      <c r="O16" s="93"/>
+      <c r="P16" s="93"/>
+      <c r="Q16" s="94"/>
+      <c r="R16" s="95"/>
+      <c r="S16" s="96"/>
+      <c r="T16" s="95"/>
+      <c r="U16" s="97"/>
+      <c r="V16" s="97"/>
+      <c r="W16" s="96"/>
+      <c r="X16" s="95"/>
+      <c r="Y16" s="96"/>
     </row>
     <row r="17" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B17" s="44"/>
-      <c r="C17" s="84"/>
-      <c r="D17" s="66"/>
-      <c r="E17" s="66"/>
-      <c r="F17" s="85"/>
-      <c r="G17" s="84"/>
-      <c r="H17" s="66"/>
-      <c r="I17" s="66"/>
-      <c r="J17" s="85"/>
-      <c r="K17" s="86"/>
-      <c r="L17" s="87"/>
-      <c r="M17" s="87"/>
-      <c r="N17" s="87"/>
-      <c r="O17" s="87"/>
-      <c r="P17" s="87"/>
-      <c r="Q17" s="88"/>
-      <c r="R17" s="84"/>
-      <c r="S17" s="85"/>
-      <c r="T17" s="84"/>
-      <c r="U17" s="66"/>
-      <c r="V17" s="66"/>
-      <c r="W17" s="85"/>
-      <c r="X17" s="84"/>
-      <c r="Y17" s="85"/>
+      <c r="C17" s="95"/>
+      <c r="D17" s="97"/>
+      <c r="E17" s="97"/>
+      <c r="F17" s="96"/>
+      <c r="G17" s="95"/>
+      <c r="H17" s="97"/>
+      <c r="I17" s="97"/>
+      <c r="J17" s="96"/>
+      <c r="K17" s="98"/>
+      <c r="L17" s="93"/>
+      <c r="M17" s="93"/>
+      <c r="N17" s="93"/>
+      <c r="O17" s="93"/>
+      <c r="P17" s="93"/>
+      <c r="Q17" s="94"/>
+      <c r="R17" s="95"/>
+      <c r="S17" s="96"/>
+      <c r="T17" s="95"/>
+      <c r="U17" s="97"/>
+      <c r="V17" s="97"/>
+      <c r="W17" s="96"/>
+      <c r="X17" s="95"/>
+      <c r="Y17" s="96"/>
     </row>
     <row r="18" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B18" s="44"/>
-      <c r="C18" s="84"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="66"/>
-      <c r="F18" s="85"/>
-      <c r="G18" s="84"/>
-      <c r="H18" s="66"/>
-      <c r="I18" s="66"/>
-      <c r="J18" s="85"/>
-      <c r="K18" s="86"/>
-      <c r="L18" s="87"/>
-      <c r="M18" s="87"/>
-      <c r="N18" s="87"/>
-      <c r="O18" s="87"/>
-      <c r="P18" s="87"/>
-      <c r="Q18" s="88"/>
-      <c r="R18" s="84"/>
-      <c r="S18" s="85"/>
-      <c r="T18" s="84"/>
-      <c r="U18" s="66"/>
-      <c r="V18" s="66"/>
-      <c r="W18" s="85"/>
-      <c r="X18" s="84"/>
-      <c r="Y18" s="85"/>
+      <c r="C18" s="95"/>
+      <c r="D18" s="97"/>
+      <c r="E18" s="97"/>
+      <c r="F18" s="96"/>
+      <c r="G18" s="95"/>
+      <c r="H18" s="97"/>
+      <c r="I18" s="97"/>
+      <c r="J18" s="96"/>
+      <c r="K18" s="98"/>
+      <c r="L18" s="93"/>
+      <c r="M18" s="93"/>
+      <c r="N18" s="93"/>
+      <c r="O18" s="93"/>
+      <c r="P18" s="93"/>
+      <c r="Q18" s="94"/>
+      <c r="R18" s="95"/>
+      <c r="S18" s="96"/>
+      <c r="T18" s="95"/>
+      <c r="U18" s="97"/>
+      <c r="V18" s="97"/>
+      <c r="W18" s="96"/>
+      <c r="X18" s="95"/>
+      <c r="Y18" s="96"/>
     </row>
     <row r="19" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B19" s="44"/>
-      <c r="C19" s="84"/>
-      <c r="D19" s="66"/>
-      <c r="E19" s="66"/>
-      <c r="F19" s="85"/>
-      <c r="G19" s="84"/>
-      <c r="H19" s="66"/>
-      <c r="I19" s="66"/>
-      <c r="J19" s="85"/>
-      <c r="K19" s="86"/>
-      <c r="L19" s="87"/>
-      <c r="M19" s="87"/>
-      <c r="N19" s="87"/>
-      <c r="O19" s="87"/>
-      <c r="P19" s="87"/>
-      <c r="Q19" s="88"/>
-      <c r="R19" s="84"/>
-      <c r="S19" s="85"/>
-      <c r="T19" s="84"/>
-      <c r="U19" s="66"/>
-      <c r="V19" s="66"/>
-      <c r="W19" s="85"/>
-      <c r="X19" s="84"/>
-      <c r="Y19" s="85"/>
+      <c r="C19" s="95"/>
+      <c r="D19" s="97"/>
+      <c r="E19" s="97"/>
+      <c r="F19" s="96"/>
+      <c r="G19" s="95"/>
+      <c r="H19" s="97"/>
+      <c r="I19" s="97"/>
+      <c r="J19" s="96"/>
+      <c r="K19" s="98"/>
+      <c r="L19" s="93"/>
+      <c r="M19" s="93"/>
+      <c r="N19" s="93"/>
+      <c r="O19" s="93"/>
+      <c r="P19" s="93"/>
+      <c r="Q19" s="94"/>
+      <c r="R19" s="95"/>
+      <c r="S19" s="96"/>
+      <c r="T19" s="95"/>
+      <c r="U19" s="97"/>
+      <c r="V19" s="97"/>
+      <c r="W19" s="96"/>
+      <c r="X19" s="95"/>
+      <c r="Y19" s="96"/>
     </row>
     <row r="20" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B20" s="44"/>
-      <c r="C20" s="84"/>
-      <c r="D20" s="66"/>
-      <c r="E20" s="66"/>
-      <c r="F20" s="85"/>
-      <c r="G20" s="84"/>
-      <c r="H20" s="66"/>
-      <c r="I20" s="66"/>
-      <c r="J20" s="85"/>
-      <c r="K20" s="86"/>
-      <c r="L20" s="87"/>
-      <c r="M20" s="87"/>
-      <c r="N20" s="87"/>
-      <c r="O20" s="87"/>
-      <c r="P20" s="87"/>
-      <c r="Q20" s="88"/>
-      <c r="R20" s="84"/>
-      <c r="S20" s="85"/>
-      <c r="T20" s="84"/>
-      <c r="U20" s="66"/>
-      <c r="V20" s="66"/>
-      <c r="W20" s="85"/>
-      <c r="X20" s="84"/>
-      <c r="Y20" s="85"/>
+      <c r="C20" s="95"/>
+      <c r="D20" s="97"/>
+      <c r="E20" s="97"/>
+      <c r="F20" s="96"/>
+      <c r="G20" s="95"/>
+      <c r="H20" s="97"/>
+      <c r="I20" s="97"/>
+      <c r="J20" s="96"/>
+      <c r="K20" s="98"/>
+      <c r="L20" s="93"/>
+      <c r="M20" s="93"/>
+      <c r="N20" s="93"/>
+      <c r="O20" s="93"/>
+      <c r="P20" s="93"/>
+      <c r="Q20" s="94"/>
+      <c r="R20" s="95"/>
+      <c r="S20" s="96"/>
+      <c r="T20" s="95"/>
+      <c r="U20" s="97"/>
+      <c r="V20" s="97"/>
+      <c r="W20" s="96"/>
+      <c r="X20" s="95"/>
+      <c r="Y20" s="96"/>
     </row>
     <row r="21" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B21" s="44"/>
-      <c r="C21" s="84"/>
-      <c r="D21" s="66"/>
-      <c r="E21" s="66"/>
-      <c r="F21" s="85"/>
-      <c r="G21" s="84"/>
-      <c r="H21" s="66"/>
-      <c r="I21" s="66"/>
-      <c r="J21" s="85"/>
-      <c r="K21" s="86"/>
-      <c r="L21" s="87"/>
-      <c r="M21" s="87"/>
-      <c r="N21" s="87"/>
-      <c r="O21" s="87"/>
-      <c r="P21" s="87"/>
-      <c r="Q21" s="88"/>
-      <c r="R21" s="84"/>
-      <c r="S21" s="85"/>
-      <c r="T21" s="84"/>
-      <c r="U21" s="66"/>
-      <c r="V21" s="66"/>
-      <c r="W21" s="85"/>
-      <c r="X21" s="84"/>
-      <c r="Y21" s="85"/>
+      <c r="C21" s="95"/>
+      <c r="D21" s="97"/>
+      <c r="E21" s="97"/>
+      <c r="F21" s="96"/>
+      <c r="G21" s="95"/>
+      <c r="H21" s="97"/>
+      <c r="I21" s="97"/>
+      <c r="J21" s="96"/>
+      <c r="K21" s="98"/>
+      <c r="L21" s="93"/>
+      <c r="M21" s="93"/>
+      <c r="N21" s="93"/>
+      <c r="O21" s="93"/>
+      <c r="P21" s="93"/>
+      <c r="Q21" s="94"/>
+      <c r="R21" s="95"/>
+      <c r="S21" s="96"/>
+      <c r="T21" s="95"/>
+      <c r="U21" s="97"/>
+      <c r="V21" s="97"/>
+      <c r="W21" s="96"/>
+      <c r="X21" s="95"/>
+      <c r="Y21" s="96"/>
     </row>
     <row r="22" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B22" s="44"/>
-      <c r="C22" s="84"/>
-      <c r="D22" s="66"/>
-      <c r="E22" s="66"/>
-      <c r="F22" s="85"/>
-      <c r="G22" s="84"/>
-      <c r="H22" s="66"/>
-      <c r="I22" s="66"/>
-      <c r="J22" s="85"/>
-      <c r="K22" s="86"/>
-      <c r="L22" s="87"/>
-      <c r="M22" s="87"/>
-      <c r="N22" s="87"/>
-      <c r="O22" s="87"/>
-      <c r="P22" s="87"/>
-      <c r="Q22" s="88"/>
-      <c r="R22" s="84"/>
-      <c r="S22" s="85"/>
-      <c r="T22" s="84"/>
-      <c r="U22" s="66"/>
-      <c r="V22" s="66"/>
-      <c r="W22" s="85"/>
-      <c r="X22" s="84"/>
-      <c r="Y22" s="85"/>
+      <c r="C22" s="95"/>
+      <c r="D22" s="97"/>
+      <c r="E22" s="97"/>
+      <c r="F22" s="96"/>
+      <c r="G22" s="95"/>
+      <c r="H22" s="97"/>
+      <c r="I22" s="97"/>
+      <c r="J22" s="96"/>
+      <c r="K22" s="98"/>
+      <c r="L22" s="93"/>
+      <c r="M22" s="93"/>
+      <c r="N22" s="93"/>
+      <c r="O22" s="93"/>
+      <c r="P22" s="93"/>
+      <c r="Q22" s="94"/>
+      <c r="R22" s="95"/>
+      <c r="S22" s="96"/>
+      <c r="T22" s="95"/>
+      <c r="U22" s="97"/>
+      <c r="V22" s="97"/>
+      <c r="W22" s="96"/>
+      <c r="X22" s="95"/>
+      <c r="Y22" s="96"/>
     </row>
     <row r="23" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B23" s="44"/>
-      <c r="C23" s="84"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="66"/>
-      <c r="F23" s="85"/>
-      <c r="G23" s="84"/>
-      <c r="H23" s="66"/>
-      <c r="I23" s="66"/>
-      <c r="J23" s="85"/>
-      <c r="K23" s="86"/>
-      <c r="L23" s="87"/>
-      <c r="M23" s="87"/>
-      <c r="N23" s="87"/>
-      <c r="O23" s="87"/>
-      <c r="P23" s="87"/>
-      <c r="Q23" s="88"/>
-      <c r="R23" s="84"/>
-      <c r="S23" s="85"/>
-      <c r="T23" s="84"/>
-      <c r="U23" s="66"/>
-      <c r="V23" s="66"/>
-      <c r="W23" s="85"/>
-      <c r="X23" s="84"/>
-      <c r="Y23" s="85"/>
+      <c r="C23" s="95"/>
+      <c r="D23" s="97"/>
+      <c r="E23" s="97"/>
+      <c r="F23" s="96"/>
+      <c r="G23" s="95"/>
+      <c r="H23" s="97"/>
+      <c r="I23" s="97"/>
+      <c r="J23" s="96"/>
+      <c r="K23" s="98"/>
+      <c r="L23" s="93"/>
+      <c r="M23" s="93"/>
+      <c r="N23" s="93"/>
+      <c r="O23" s="93"/>
+      <c r="P23" s="93"/>
+      <c r="Q23" s="94"/>
+      <c r="R23" s="95"/>
+      <c r="S23" s="96"/>
+      <c r="T23" s="95"/>
+      <c r="U23" s="97"/>
+      <c r="V23" s="97"/>
+      <c r="W23" s="96"/>
+      <c r="X23" s="95"/>
+      <c r="Y23" s="96"/>
     </row>
     <row r="24" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B24" s="44"/>
-      <c r="C24" s="84"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="66"/>
-      <c r="F24" s="85"/>
-      <c r="G24" s="84"/>
-      <c r="H24" s="66"/>
-      <c r="I24" s="66"/>
-      <c r="J24" s="85"/>
-      <c r="K24" s="86"/>
-      <c r="L24" s="87"/>
-      <c r="M24" s="87"/>
-      <c r="N24" s="87"/>
-      <c r="O24" s="87"/>
-      <c r="P24" s="87"/>
-      <c r="Q24" s="88"/>
-      <c r="R24" s="84"/>
-      <c r="S24" s="85"/>
-      <c r="T24" s="84"/>
-      <c r="U24" s="66"/>
-      <c r="V24" s="66"/>
-      <c r="W24" s="85"/>
-      <c r="X24" s="84"/>
-      <c r="Y24" s="85"/>
+      <c r="C24" s="95"/>
+      <c r="D24" s="97"/>
+      <c r="E24" s="97"/>
+      <c r="F24" s="96"/>
+      <c r="G24" s="95"/>
+      <c r="H24" s="97"/>
+      <c r="I24" s="97"/>
+      <c r="J24" s="96"/>
+      <c r="K24" s="98"/>
+      <c r="L24" s="93"/>
+      <c r="M24" s="93"/>
+      <c r="N24" s="93"/>
+      <c r="O24" s="93"/>
+      <c r="P24" s="93"/>
+      <c r="Q24" s="94"/>
+      <c r="R24" s="95"/>
+      <c r="S24" s="96"/>
+      <c r="T24" s="95"/>
+      <c r="U24" s="97"/>
+      <c r="V24" s="97"/>
+      <c r="W24" s="96"/>
+      <c r="X24" s="95"/>
+      <c r="Y24" s="96"/>
     </row>
     <row r="25" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B25" s="44"/>
-      <c r="C25" s="84"/>
-      <c r="D25" s="66"/>
-      <c r="E25" s="66"/>
-      <c r="F25" s="85"/>
-      <c r="G25" s="84"/>
-      <c r="H25" s="66"/>
-      <c r="I25" s="66"/>
-      <c r="J25" s="85"/>
-      <c r="K25" s="86"/>
-      <c r="L25" s="87"/>
-      <c r="M25" s="87"/>
-      <c r="N25" s="87"/>
-      <c r="O25" s="87"/>
-      <c r="P25" s="87"/>
-      <c r="Q25" s="88"/>
-      <c r="R25" s="84"/>
-      <c r="S25" s="85"/>
-      <c r="T25" s="84"/>
-      <c r="U25" s="66"/>
-      <c r="V25" s="66"/>
-      <c r="W25" s="85"/>
-      <c r="X25" s="84"/>
-      <c r="Y25" s="85"/>
+      <c r="C25" s="95"/>
+      <c r="D25" s="97"/>
+      <c r="E25" s="97"/>
+      <c r="F25" s="96"/>
+      <c r="G25" s="95"/>
+      <c r="H25" s="97"/>
+      <c r="I25" s="97"/>
+      <c r="J25" s="96"/>
+      <c r="K25" s="98"/>
+      <c r="L25" s="93"/>
+      <c r="M25" s="93"/>
+      <c r="N25" s="93"/>
+      <c r="O25" s="93"/>
+      <c r="P25" s="93"/>
+      <c r="Q25" s="94"/>
+      <c r="R25" s="95"/>
+      <c r="S25" s="96"/>
+      <c r="T25" s="95"/>
+      <c r="U25" s="97"/>
+      <c r="V25" s="97"/>
+      <c r="W25" s="96"/>
+      <c r="X25" s="95"/>
+      <c r="Y25" s="96"/>
     </row>
     <row r="26" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B26" s="44"/>
-      <c r="C26" s="84"/>
-      <c r="D26" s="66"/>
-      <c r="E26" s="66"/>
-      <c r="F26" s="85"/>
-      <c r="G26" s="84"/>
-      <c r="H26" s="66"/>
-      <c r="I26" s="66"/>
-      <c r="J26" s="85"/>
-      <c r="K26" s="86"/>
-      <c r="L26" s="87"/>
-      <c r="M26" s="87"/>
-      <c r="N26" s="87"/>
-      <c r="O26" s="87"/>
-      <c r="P26" s="87"/>
-      <c r="Q26" s="88"/>
-      <c r="R26" s="84"/>
-      <c r="S26" s="85"/>
-      <c r="T26" s="84"/>
-      <c r="U26" s="66"/>
-      <c r="V26" s="66"/>
-      <c r="W26" s="85"/>
-      <c r="X26" s="84"/>
-      <c r="Y26" s="85"/>
+      <c r="C26" s="95"/>
+      <c r="D26" s="97"/>
+      <c r="E26" s="97"/>
+      <c r="F26" s="96"/>
+      <c r="G26" s="95"/>
+      <c r="H26" s="97"/>
+      <c r="I26" s="97"/>
+      <c r="J26" s="96"/>
+      <c r="K26" s="98"/>
+      <c r="L26" s="93"/>
+      <c r="M26" s="93"/>
+      <c r="N26" s="93"/>
+      <c r="O26" s="93"/>
+      <c r="P26" s="93"/>
+      <c r="Q26" s="94"/>
+      <c r="R26" s="95"/>
+      <c r="S26" s="96"/>
+      <c r="T26" s="95"/>
+      <c r="U26" s="97"/>
+      <c r="V26" s="97"/>
+      <c r="W26" s="96"/>
+      <c r="X26" s="95"/>
+      <c r="Y26" s="96"/>
     </row>
     <row r="27" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B27" s="44"/>
-      <c r="C27" s="84"/>
-      <c r="D27" s="66"/>
-      <c r="E27" s="66"/>
-      <c r="F27" s="85"/>
-      <c r="G27" s="84"/>
-      <c r="H27" s="66"/>
-      <c r="I27" s="66"/>
-      <c r="J27" s="85"/>
-      <c r="K27" s="86"/>
-      <c r="L27" s="87"/>
-      <c r="M27" s="87"/>
-      <c r="N27" s="87"/>
-      <c r="O27" s="87"/>
-      <c r="P27" s="87"/>
-      <c r="Q27" s="88"/>
-      <c r="R27" s="84"/>
-      <c r="S27" s="85"/>
-      <c r="T27" s="84"/>
-      <c r="U27" s="66"/>
-      <c r="V27" s="66"/>
-      <c r="W27" s="85"/>
-      <c r="X27" s="84"/>
-      <c r="Y27" s="85"/>
+      <c r="C27" s="95"/>
+      <c r="D27" s="97"/>
+      <c r="E27" s="97"/>
+      <c r="F27" s="96"/>
+      <c r="G27" s="95"/>
+      <c r="H27" s="97"/>
+      <c r="I27" s="97"/>
+      <c r="J27" s="96"/>
+      <c r="K27" s="98"/>
+      <c r="L27" s="93"/>
+      <c r="M27" s="93"/>
+      <c r="N27" s="93"/>
+      <c r="O27" s="93"/>
+      <c r="P27" s="93"/>
+      <c r="Q27" s="94"/>
+      <c r="R27" s="95"/>
+      <c r="S27" s="96"/>
+      <c r="T27" s="95"/>
+      <c r="U27" s="97"/>
+      <c r="V27" s="97"/>
+      <c r="W27" s="96"/>
+      <c r="X27" s="95"/>
+      <c r="Y27" s="96"/>
     </row>
     <row r="28" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B28" s="44"/>
-      <c r="C28" s="84"/>
-      <c r="D28" s="66"/>
-      <c r="E28" s="66"/>
-      <c r="F28" s="85"/>
-      <c r="G28" s="84"/>
-      <c r="H28" s="66"/>
-      <c r="I28" s="66"/>
-      <c r="J28" s="85"/>
-      <c r="K28" s="86"/>
-      <c r="L28" s="87"/>
-      <c r="M28" s="87"/>
-      <c r="N28" s="87"/>
-      <c r="O28" s="87"/>
-      <c r="P28" s="87"/>
-      <c r="Q28" s="88"/>
-      <c r="R28" s="84"/>
-      <c r="S28" s="85"/>
-      <c r="T28" s="84"/>
-      <c r="U28" s="66"/>
-      <c r="V28" s="66"/>
-      <c r="W28" s="85"/>
-      <c r="X28" s="84"/>
-      <c r="Y28" s="85"/>
+      <c r="C28" s="95"/>
+      <c r="D28" s="97"/>
+      <c r="E28" s="97"/>
+      <c r="F28" s="96"/>
+      <c r="G28" s="95"/>
+      <c r="H28" s="97"/>
+      <c r="I28" s="97"/>
+      <c r="J28" s="96"/>
+      <c r="K28" s="98"/>
+      <c r="L28" s="93"/>
+      <c r="M28" s="93"/>
+      <c r="N28" s="93"/>
+      <c r="O28" s="93"/>
+      <c r="P28" s="93"/>
+      <c r="Q28" s="94"/>
+      <c r="R28" s="95"/>
+      <c r="S28" s="96"/>
+      <c r="T28" s="95"/>
+      <c r="U28" s="97"/>
+      <c r="V28" s="97"/>
+      <c r="W28" s="96"/>
+      <c r="X28" s="95"/>
+      <c r="Y28" s="96"/>
     </row>
     <row r="29" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B29" s="44"/>
-      <c r="C29" s="84"/>
-      <c r="D29" s="66"/>
-      <c r="E29" s="66"/>
-      <c r="F29" s="85"/>
-      <c r="G29" s="84"/>
-      <c r="H29" s="66"/>
-      <c r="I29" s="66"/>
-      <c r="J29" s="85"/>
-      <c r="K29" s="86"/>
-      <c r="L29" s="87"/>
-      <c r="M29" s="87"/>
-      <c r="N29" s="87"/>
-      <c r="O29" s="87"/>
-      <c r="P29" s="87"/>
-      <c r="Q29" s="88"/>
-      <c r="R29" s="84"/>
-      <c r="S29" s="85"/>
-      <c r="T29" s="84"/>
-      <c r="U29" s="66"/>
-      <c r="V29" s="66"/>
-      <c r="W29" s="85"/>
-      <c r="X29" s="84"/>
-      <c r="Y29" s="85"/>
+      <c r="C29" s="95"/>
+      <c r="D29" s="97"/>
+      <c r="E29" s="97"/>
+      <c r="F29" s="96"/>
+      <c r="G29" s="95"/>
+      <c r="H29" s="97"/>
+      <c r="I29" s="97"/>
+      <c r="J29" s="96"/>
+      <c r="K29" s="98"/>
+      <c r="L29" s="93"/>
+      <c r="M29" s="93"/>
+      <c r="N29" s="93"/>
+      <c r="O29" s="93"/>
+      <c r="P29" s="93"/>
+      <c r="Q29" s="94"/>
+      <c r="R29" s="95"/>
+      <c r="S29" s="96"/>
+      <c r="T29" s="95"/>
+      <c r="U29" s="97"/>
+      <c r="V29" s="97"/>
+      <c r="W29" s="96"/>
+      <c r="X29" s="95"/>
+      <c r="Y29" s="96"/>
     </row>
     <row r="30" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B30" s="44"/>
-      <c r="C30" s="84"/>
-      <c r="D30" s="66"/>
-      <c r="E30" s="66"/>
-      <c r="F30" s="85"/>
-      <c r="G30" s="84"/>
-      <c r="H30" s="66"/>
-      <c r="I30" s="66"/>
-      <c r="J30" s="85"/>
-      <c r="K30" s="86"/>
-      <c r="L30" s="87"/>
-      <c r="M30" s="87"/>
-      <c r="N30" s="87"/>
-      <c r="O30" s="87"/>
-      <c r="P30" s="87"/>
-      <c r="Q30" s="88"/>
-      <c r="R30" s="84"/>
-      <c r="S30" s="85"/>
-      <c r="T30" s="84"/>
-      <c r="U30" s="66"/>
-      <c r="V30" s="66"/>
-      <c r="W30" s="85"/>
-      <c r="X30" s="84"/>
-      <c r="Y30" s="85"/>
+      <c r="C30" s="95"/>
+      <c r="D30" s="97"/>
+      <c r="E30" s="97"/>
+      <c r="F30" s="96"/>
+      <c r="G30" s="95"/>
+      <c r="H30" s="97"/>
+      <c r="I30" s="97"/>
+      <c r="J30" s="96"/>
+      <c r="K30" s="98"/>
+      <c r="L30" s="93"/>
+      <c r="M30" s="93"/>
+      <c r="N30" s="93"/>
+      <c r="O30" s="93"/>
+      <c r="P30" s="93"/>
+      <c r="Q30" s="94"/>
+      <c r="R30" s="95"/>
+      <c r="S30" s="96"/>
+      <c r="T30" s="95"/>
+      <c r="U30" s="97"/>
+      <c r="V30" s="97"/>
+      <c r="W30" s="96"/>
+      <c r="X30" s="95"/>
+      <c r="Y30" s="96"/>
     </row>
     <row r="31" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="43"/>
       <c r="B31" s="44"/>
-      <c r="C31" s="89"/>
-      <c r="D31" s="90"/>
-      <c r="E31" s="90"/>
-      <c r="F31" s="91"/>
-      <c r="G31" s="89"/>
-      <c r="H31" s="90"/>
-      <c r="I31" s="90"/>
-      <c r="J31" s="91"/>
-      <c r="K31" s="86"/>
-      <c r="L31" s="87"/>
-      <c r="M31" s="87"/>
-      <c r="N31" s="87"/>
-      <c r="O31" s="87"/>
-      <c r="P31" s="87"/>
-      <c r="Q31" s="88"/>
-      <c r="R31" s="84"/>
-      <c r="S31" s="85"/>
-      <c r="T31" s="84"/>
-      <c r="U31" s="66"/>
-      <c r="V31" s="66"/>
-      <c r="W31" s="85"/>
-      <c r="X31" s="84"/>
-      <c r="Y31" s="85"/>
+      <c r="C31" s="83"/>
+      <c r="D31" s="84"/>
+      <c r="E31" s="84"/>
+      <c r="F31" s="85"/>
+      <c r="G31" s="83"/>
+      <c r="H31" s="84"/>
+      <c r="I31" s="84"/>
+      <c r="J31" s="85"/>
+      <c r="K31" s="98"/>
+      <c r="L31" s="93"/>
+      <c r="M31" s="93"/>
+      <c r="N31" s="93"/>
+      <c r="O31" s="93"/>
+      <c r="P31" s="93"/>
+      <c r="Q31" s="94"/>
+      <c r="R31" s="95"/>
+      <c r="S31" s="96"/>
+      <c r="T31" s="95"/>
+      <c r="U31" s="97"/>
+      <c r="V31" s="97"/>
+      <c r="W31" s="96"/>
+      <c r="X31" s="95"/>
+      <c r="Y31" s="96"/>
     </row>
     <row r="32" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="43"/>
       <c r="B32" s="44"/>
-      <c r="C32" s="89"/>
-      <c r="D32" s="90"/>
-      <c r="E32" s="90"/>
-      <c r="F32" s="91"/>
-      <c r="G32" s="89"/>
-      <c r="H32" s="90"/>
-      <c r="I32" s="90"/>
-      <c r="J32" s="91"/>
+      <c r="C32" s="83"/>
+      <c r="D32" s="84"/>
+      <c r="E32" s="84"/>
+      <c r="F32" s="85"/>
+      <c r="G32" s="83"/>
+      <c r="H32" s="84"/>
+      <c r="I32" s="84"/>
+      <c r="J32" s="85"/>
       <c r="K32" s="92"/>
-      <c r="L32" s="87"/>
-      <c r="M32" s="87"/>
-      <c r="N32" s="87"/>
-      <c r="O32" s="87"/>
-      <c r="P32" s="87"/>
-      <c r="Q32" s="88"/>
-      <c r="R32" s="84"/>
-      <c r="S32" s="85"/>
-      <c r="T32" s="84"/>
-      <c r="U32" s="66"/>
-      <c r="V32" s="66"/>
-      <c r="W32" s="85"/>
-      <c r="X32" s="84"/>
-      <c r="Y32" s="85"/>
+      <c r="L32" s="93"/>
+      <c r="M32" s="93"/>
+      <c r="N32" s="93"/>
+      <c r="O32" s="93"/>
+      <c r="P32" s="93"/>
+      <c r="Q32" s="94"/>
+      <c r="R32" s="95"/>
+      <c r="S32" s="96"/>
+      <c r="T32" s="95"/>
+      <c r="U32" s="97"/>
+      <c r="V32" s="97"/>
+      <c r="W32" s="96"/>
+      <c r="X32" s="95"/>
+      <c r="Y32" s="96"/>
     </row>
     <row r="33" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="45"/>
       <c r="B33" s="46"/>
-      <c r="C33" s="89"/>
-      <c r="D33" s="90"/>
-      <c r="E33" s="90"/>
-      <c r="F33" s="91"/>
-      <c r="G33" s="89"/>
-      <c r="H33" s="90"/>
-      <c r="I33" s="90"/>
-      <c r="J33" s="91"/>
-      <c r="K33" s="110"/>
-      <c r="L33" s="111"/>
-      <c r="M33" s="111"/>
-      <c r="N33" s="111"/>
-      <c r="O33" s="111"/>
-      <c r="P33" s="111"/>
-      <c r="Q33" s="112"/>
-      <c r="R33" s="113"/>
-      <c r="S33" s="114"/>
-      <c r="T33" s="113"/>
-      <c r="U33" s="115"/>
-      <c r="V33" s="115"/>
-      <c r="W33" s="114"/>
-      <c r="X33" s="113"/>
-      <c r="Y33" s="114"/>
+      <c r="C33" s="83"/>
+      <c r="D33" s="84"/>
+      <c r="E33" s="84"/>
+      <c r="F33" s="85"/>
+      <c r="G33" s="83"/>
+      <c r="H33" s="84"/>
+      <c r="I33" s="84"/>
+      <c r="J33" s="85"/>
+      <c r="K33" s="86"/>
+      <c r="L33" s="87"/>
+      <c r="M33" s="87"/>
+      <c r="N33" s="87"/>
+      <c r="O33" s="87"/>
+      <c r="P33" s="87"/>
+      <c r="Q33" s="88"/>
+      <c r="R33" s="89"/>
+      <c r="S33" s="90"/>
+      <c r="T33" s="89"/>
+      <c r="U33" s="91"/>
+      <c r="V33" s="91"/>
+      <c r="W33" s="90"/>
+      <c r="X33" s="89"/>
+      <c r="Y33" s="90"/>
     </row>
     <row r="34" spans="1:25" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="93" t="s">
+      <c r="A34" s="66" t="s">
         <v>361</v>
       </c>
-      <c r="B34" s="94"/>
-      <c r="C34" s="97" t="s">
+      <c r="B34" s="67"/>
+      <c r="C34" s="70" t="s">
         <v>362</v>
       </c>
-      <c r="D34" s="98"/>
-      <c r="E34" s="98"/>
-      <c r="F34" s="99"/>
-      <c r="G34" s="97" t="s">
+      <c r="D34" s="71"/>
+      <c r="E34" s="71"/>
+      <c r="F34" s="72"/>
+      <c r="G34" s="70" t="s">
         <v>363</v>
       </c>
-      <c r="H34" s="98"/>
-      <c r="I34" s="98"/>
-      <c r="J34" s="99"/>
-      <c r="K34" s="93" t="s">
+      <c r="H34" s="71"/>
+      <c r="I34" s="71"/>
+      <c r="J34" s="72"/>
+      <c r="K34" s="66" t="s">
         <v>364</v>
       </c>
-      <c r="L34" s="103"/>
-      <c r="M34" s="103"/>
-      <c r="N34" s="103"/>
-      <c r="O34" s="103"/>
-      <c r="P34" s="103"/>
-      <c r="Q34" s="104"/>
-      <c r="R34" s="93" t="s">
+      <c r="L34" s="76"/>
+      <c r="M34" s="76"/>
+      <c r="N34" s="76"/>
+      <c r="O34" s="76"/>
+      <c r="P34" s="76"/>
+      <c r="Q34" s="77"/>
+      <c r="R34" s="66" t="s">
         <v>365</v>
       </c>
-      <c r="S34" s="94"/>
-      <c r="T34" s="93" t="s">
+      <c r="S34" s="67"/>
+      <c r="T34" s="66" t="s">
         <v>366</v>
       </c>
-      <c r="U34" s="108"/>
-      <c r="V34" s="108"/>
-      <c r="W34" s="94"/>
-      <c r="X34" s="93" t="s">
+      <c r="U34" s="81"/>
+      <c r="V34" s="81"/>
+      <c r="W34" s="67"/>
+      <c r="X34" s="66" t="s">
         <v>367</v>
       </c>
-      <c r="Y34" s="94"/>
+      <c r="Y34" s="67"/>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A35" s="95"/>
-      <c r="B35" s="96"/>
-      <c r="C35" s="100"/>
-      <c r="D35" s="101"/>
-      <c r="E35" s="101"/>
-      <c r="F35" s="102"/>
-      <c r="G35" s="100"/>
-      <c r="H35" s="101"/>
-      <c r="I35" s="101"/>
-      <c r="J35" s="102"/>
-      <c r="K35" s="105"/>
-      <c r="L35" s="106"/>
-      <c r="M35" s="106"/>
-      <c r="N35" s="106"/>
-      <c r="O35" s="106"/>
-      <c r="P35" s="106"/>
-      <c r="Q35" s="107"/>
-      <c r="R35" s="95"/>
-      <c r="S35" s="96"/>
-      <c r="T35" s="95"/>
-      <c r="U35" s="109"/>
-      <c r="V35" s="109"/>
-      <c r="W35" s="96"/>
-      <c r="X35" s="95"/>
-      <c r="Y35" s="96"/>
+      <c r="A35" s="68"/>
+      <c r="B35" s="69"/>
+      <c r="C35" s="73"/>
+      <c r="D35" s="74"/>
+      <c r="E35" s="74"/>
+      <c r="F35" s="75"/>
+      <c r="G35" s="73"/>
+      <c r="H35" s="74"/>
+      <c r="I35" s="74"/>
+      <c r="J35" s="75"/>
+      <c r="K35" s="78"/>
+      <c r="L35" s="79"/>
+      <c r="M35" s="79"/>
+      <c r="N35" s="79"/>
+      <c r="O35" s="79"/>
+      <c r="P35" s="79"/>
+      <c r="Q35" s="80"/>
+      <c r="R35" s="68"/>
+      <c r="S35" s="69"/>
+      <c r="T35" s="68"/>
+      <c r="U35" s="82"/>
+      <c r="V35" s="82"/>
+      <c r="W35" s="69"/>
+      <c r="X35" s="68"/>
+      <c r="Y35" s="69"/>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A36" s="47" t="s">
@@ -11938,116 +11938,15 @@
     </row>
   </sheetData>
   <mergeCells count="143">
-    <mergeCell ref="X34:Y35"/>
-    <mergeCell ref="A34:B35"/>
-    <mergeCell ref="C34:F35"/>
-    <mergeCell ref="G34:J35"/>
-    <mergeCell ref="K34:Q35"/>
-    <mergeCell ref="R34:S35"/>
-    <mergeCell ref="T34:W35"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="K33:Q33"/>
-    <mergeCell ref="R33:S33"/>
-    <mergeCell ref="T33:W33"/>
-    <mergeCell ref="X33:Y33"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="K32:Q32"/>
-    <mergeCell ref="R32:S32"/>
-    <mergeCell ref="T32:W32"/>
-    <mergeCell ref="X32:Y32"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K31:Q31"/>
-    <mergeCell ref="R31:S31"/>
-    <mergeCell ref="T31:W31"/>
-    <mergeCell ref="X31:Y31"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="K30:Q30"/>
-    <mergeCell ref="R30:S30"/>
-    <mergeCell ref="T30:W30"/>
-    <mergeCell ref="X30:Y30"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="K29:Q29"/>
-    <mergeCell ref="R29:S29"/>
-    <mergeCell ref="T29:W29"/>
-    <mergeCell ref="X29:Y29"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="K28:Q28"/>
-    <mergeCell ref="R28:S28"/>
-    <mergeCell ref="T28:W28"/>
-    <mergeCell ref="X28:Y28"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="K27:Q27"/>
-    <mergeCell ref="R27:S27"/>
-    <mergeCell ref="T27:W27"/>
-    <mergeCell ref="X27:Y27"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="K26:Q26"/>
-    <mergeCell ref="R26:S26"/>
-    <mergeCell ref="T26:W26"/>
-    <mergeCell ref="X26:Y26"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="K25:Q25"/>
-    <mergeCell ref="R25:S25"/>
-    <mergeCell ref="T25:W25"/>
-    <mergeCell ref="X25:Y25"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K24:Q24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="T24:W24"/>
-    <mergeCell ref="X24:Y24"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="K23:Q23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="T23:W23"/>
-    <mergeCell ref="X23:Y23"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="G22:J22"/>
-    <mergeCell ref="K22:Q22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="T22:W22"/>
-    <mergeCell ref="X22:Y22"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K21:Q21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="T21:W21"/>
-    <mergeCell ref="X21:Y21"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="K20:Q20"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="T20:W20"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="K19:Q19"/>
-    <mergeCell ref="R19:S19"/>
-    <mergeCell ref="T19:W19"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="T14:W14"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="K18:Q18"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="T18:W18"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="K17:Q17"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="T17:W17"/>
-    <mergeCell ref="X17:Y17"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="O7:Q8"/>
+    <mergeCell ref="R7:T8"/>
+    <mergeCell ref="U7:W8"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="S10:W10"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="S11:W11"/>
+    <mergeCell ref="P1:V1"/>
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="D2:W2"/>
     <mergeCell ref="D3:W3"/>
@@ -12072,15 +11971,116 @@
     <mergeCell ref="G14:J14"/>
     <mergeCell ref="K14:Q14"/>
     <mergeCell ref="R14:S14"/>
-    <mergeCell ref="P12:R12"/>
-    <mergeCell ref="O7:Q8"/>
-    <mergeCell ref="R7:T8"/>
-    <mergeCell ref="U7:W8"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="S10:W10"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="S11:W11"/>
-    <mergeCell ref="P1:V1"/>
+    <mergeCell ref="T14:W14"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="K18:Q18"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="T18:W18"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="K17:Q17"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="T17:W17"/>
+    <mergeCell ref="X17:Y17"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="K20:Q20"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="T20:W20"/>
+    <mergeCell ref="X20:Y20"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="K19:Q19"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="T19:W19"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="K22:Q22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="T22:W22"/>
+    <mergeCell ref="X22:Y22"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K21:Q21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="T21:W21"/>
+    <mergeCell ref="X21:Y21"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K24:Q24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="T24:W24"/>
+    <mergeCell ref="X24:Y24"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="K23:Q23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="T23:W23"/>
+    <mergeCell ref="X23:Y23"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="K26:Q26"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="T26:W26"/>
+    <mergeCell ref="X26:Y26"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="K25:Q25"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="T25:W25"/>
+    <mergeCell ref="X25:Y25"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="K28:Q28"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="T28:W28"/>
+    <mergeCell ref="X28:Y28"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="K27:Q27"/>
+    <mergeCell ref="R27:S27"/>
+    <mergeCell ref="T27:W27"/>
+    <mergeCell ref="X27:Y27"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="K30:Q30"/>
+    <mergeCell ref="R30:S30"/>
+    <mergeCell ref="T30:W30"/>
+    <mergeCell ref="X30:Y30"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="K29:Q29"/>
+    <mergeCell ref="R29:S29"/>
+    <mergeCell ref="T29:W29"/>
+    <mergeCell ref="X29:Y29"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="K32:Q32"/>
+    <mergeCell ref="R32:S32"/>
+    <mergeCell ref="T32:W32"/>
+    <mergeCell ref="X32:Y32"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K31:Q31"/>
+    <mergeCell ref="R31:S31"/>
+    <mergeCell ref="T31:W31"/>
+    <mergeCell ref="X31:Y31"/>
+    <mergeCell ref="X34:Y35"/>
+    <mergeCell ref="A34:B35"/>
+    <mergeCell ref="C34:F35"/>
+    <mergeCell ref="G34:J35"/>
+    <mergeCell ref="K34:Q35"/>
+    <mergeCell ref="R34:S35"/>
+    <mergeCell ref="T34:W35"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="K33:Q33"/>
+    <mergeCell ref="R33:S33"/>
+    <mergeCell ref="T33:W33"/>
+    <mergeCell ref="X33:Y33"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.86614173228346458" right="0.51181102362204722" top="0.59055118110236227" bottom="0.19685039370078741" header="0.59055118110236227" footer="0.19685039370078741"/>

</xml_diff>

<commit_message>
sync(workvault): 2026-10-26 18:38 差分 2 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/LNB管理手順書案_未承認.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/LNB管理手順書案_未承認.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nk365-my.sharepoint.com/personal/ss80751_ad_nkc_co_jp/Documents/ドキュメント/Work_Vault/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="6_{C0F3EAFA-DEEC-4CD0-B5EF-21988F4F198C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E526E21C-A2AF-49D8-835E-6CDF4B701051}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="6_{C0F3EAFA-DEEC-4CD0-B5EF-21988F4F198C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1BA0FD4-6038-4310-B888-CC80A25024F8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
     <sheet name="引用と部品照合" sheetId="17" r:id="rId17"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">相関図!$A$1:$AY$55</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">相関図!$A$1:$AY$58</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">定期管理!$A$1:$AZ$100</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="12">'チェックシート(月次・異常時)'!$1:$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'チェックシート(日次)'!$1:$3</definedName>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="389">
   <si>
     <t>手 順 書</t>
   </si>
@@ -1453,10 +1453,16 @@
     <t>確定事項のみ記載。出典：公式資料・操作手順書 0494-912039(06)・会議記録。暫定・未確認の経路は含まない</t>
   </si>
   <si>
-    <t>凡例：【サーバ】=サーバー(VM含む)／【端末(PC)】=作業員が操作するPC／【設備】=製造設備／【表示】=画面・表示装置／【保存領域】=ファイル保存場所。色: 青=サーバ・表示系／黄=PC・操作端末／緑=設備・データ保存</t>
-  </si>
-  <si>
-    <t>配置：A4 縦 1 頁。事象別の図(アンドン・稼働モニタ異常／月次再起動／異常時再起動)は PanaCIM_LNB_確実構成図.drawio に残置。</t>
+    <t>凡例：【サーバ】=サーバー(VM含む)／【端末(PC)】=作業員が操作するPC／【設備】=製造設備／【表示】=画面・表示装置</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>　　　【保存領域】=ファイル保存場所。色: 青=サーバ・表示系／黄=PC・操作端末／緑=設備・データ保存</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>配置：A4縦1頁。事象別の図(アンドン・稼働モニタ異常/月次再起動/異常時再起動)は確実構成図.drawioに残置</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -6477,13 +6483,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>119380</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>127000</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>104140</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6554,13 +6560,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>119380</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>96520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>127000</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>142240</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6631,13 +6637,13 @@
     <xdr:from>
       <xdr:col>27</xdr:col>
       <xdr:colOff>20320</xdr:colOff>
-      <xdr:row>9</xdr:row>
+      <xdr:row>10</xdr:row>
       <xdr:rowOff>15240</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>50</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>33020</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6708,13 +6714,13 @@
     <xdr:from>
       <xdr:col>27</xdr:col>
       <xdr:colOff>20320</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>25400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>50</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>142240</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6762,10 +6768,10 @@
         </a:fontRef>
       </xdr:style>
       <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="50800" tIns="25400" rIns="76200" bIns="12700" rtlCol="0" anchor="t" anchorCtr="1"/>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" lIns="25400" tIns="25400" rIns="76200" bIns="12700" rtlCol="0" anchor="t" anchorCtr="0"/>
         <a:lstStyle/>
         <a:p>
-          <a:pPr algn="l"/>
+          <a:pPr algn="r"/>
           <a:r>
             <a:rPr kumimoji="1" lang="ja-JP" altLang="en-US" sz="800" b="1">
               <a:solidFill>
@@ -6805,13 +6811,13 @@
     <xdr:from>
       <xdr:col>27</xdr:col>
       <xdr:colOff>20320</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>31</xdr:row>
       <xdr:rowOff>134620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>50</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>39</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6882,13 +6888,13 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>119380</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>41</xdr:row>
       <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>50</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>49</xdr:row>
+      <xdr:row>50</xdr:row>
       <xdr:rowOff>40640</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -6979,13 +6985,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>116840</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>45720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>73660</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7086,13 +7092,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>116840</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>5080</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>149860</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7253,13 +7259,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>40640</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>10160</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7417,13 +7423,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>111760</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>27</xdr:row>
+      <xdr:row>28</xdr:row>
       <xdr:rowOff>157480</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7571,13 +7577,13 @@
     <xdr:from>
       <xdr:col>28</xdr:col>
       <xdr:colOff>17780</xdr:colOff>
-      <xdr:row>10</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>134620</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>49</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>27940</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7698,13 +7704,13 @@
     <xdr:from>
       <xdr:col>28</xdr:col>
       <xdr:colOff>17780</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>20320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>49</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>149860</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7825,13 +7831,13 @@
     <xdr:from>
       <xdr:col>28</xdr:col>
       <xdr:colOff>17780</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>119380</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>38</xdr:col>
       <xdr:colOff>93980</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>121920</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -7952,13 +7958,13 @@
     <xdr:from>
       <xdr:col>39</xdr:col>
       <xdr:colOff>66040</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>119380</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>49</xdr:col>
       <xdr:colOff>116840</xdr:colOff>
-      <xdr:row>25</xdr:row>
+      <xdr:row>26</xdr:row>
       <xdr:rowOff>121920</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -8059,13 +8065,13 @@
     <xdr:from>
       <xdr:col>28</xdr:col>
       <xdr:colOff>17780</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>119380</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>49</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>38</xdr:row>
       <xdr:rowOff>5080</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -8183,14 +8189,14 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>12700</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>17780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>20320</xdr:rowOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -8206,7 +8212,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="660400" y="7416800"/>
-          <a:ext cx="1397000" cy="482600"/>
+          <a:ext cx="1397000" cy="762000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -8310,14 +8316,14 @@
     <xdr:from>
       <xdr:col>16</xdr:col>
       <xdr:colOff>86360</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>17780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>27</xdr:col>
       <xdr:colOff>58420</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>20320</xdr:rowOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>139700</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -8333,7 +8339,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="2159000" y="7416800"/>
-          <a:ext cx="1397000" cy="482600"/>
+          <a:ext cx="1397000" cy="762000"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -8437,14 +8443,14 @@
     <xdr:from>
       <xdr:col>3</xdr:col>
       <xdr:colOff>119380</xdr:colOff>
-      <xdr:row>50</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>33020</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>50</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>104140</xdr:rowOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>81280</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -8460,7 +8466,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="508000" y="8712200"/>
-          <a:ext cx="5969000" cy="711200"/>
+          <a:ext cx="5969000" cy="1168400"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -8794,13 +8800,13 @@
     <xdr:from>
       <xdr:col>14</xdr:col>
       <xdr:colOff>123190</xdr:colOff>
-      <xdr:row>13</xdr:row>
+      <xdr:row>14</xdr:row>
       <xdr:rowOff>73660</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
       <xdr:colOff>123190</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>40640</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -8850,13 +8856,13 @@
     <xdr:from>
       <xdr:col>15</xdr:col>
       <xdr:colOff>63500</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>96520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>21</xdr:col>
       <xdr:colOff>48260</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -8941,13 +8947,13 @@
     <xdr:from>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>13</xdr:row>
       <xdr:rowOff>81280</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>17780</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>66040</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -8997,13 +9003,13 @@
     <xdr:from>
       <xdr:col>21</xdr:col>
       <xdr:colOff>99060</xdr:colOff>
-      <xdr:row>15</xdr:row>
+      <xdr:row>16</xdr:row>
       <xdr:rowOff>96520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>88900</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>17</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -9088,13 +9094,13 @@
     <xdr:from>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>28</xdr:col>
       <xdr:colOff>17780</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>35</xdr:row>
       <xdr:rowOff>142240</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -9145,13 +9151,13 @@
       <xdr:col>19</xdr:col>
       <xdr:colOff>78740</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>12700</xdr:rowOff>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>26</xdr:col>
       <xdr:colOff>35560</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -9166,8 +9172,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2540000" y="5651500"/>
-          <a:ext cx="863600" cy="139700"/>
+          <a:off x="2540000" y="5562600"/>
+          <a:ext cx="863600" cy="381000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9255,13 +9261,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>63500</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>149860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>60960</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>17780</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -9311,13 +9317,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>38</xdr:row>
       <xdr:rowOff>106680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
       <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>86360</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -9412,13 +9418,13 @@
     <xdr:from>
       <xdr:col>19</xdr:col>
       <xdr:colOff>15240</xdr:colOff>
-      <xdr:row>28</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>149860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
       <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>42</xdr:row>
+      <xdr:row>43</xdr:row>
       <xdr:rowOff>17780</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -9468,13 +9474,13 @@
     <xdr:from>
       <xdr:col>23</xdr:col>
       <xdr:colOff>68580</xdr:colOff>
-      <xdr:row>37</xdr:row>
+      <xdr:row>38</xdr:row>
       <xdr:rowOff>144780</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>25</xdr:col>
       <xdr:colOff>88900</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>39</xdr:row>
       <xdr:rowOff>124460</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -9559,13 +9565,13 @@
     <xdr:from>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>33</xdr:col>
       <xdr:colOff>55880</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>119380</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -9615,13 +9621,13 @@
     <xdr:from>
       <xdr:col>35</xdr:col>
       <xdr:colOff>63500</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>25400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>39</xdr:col>
       <xdr:colOff>104140</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>5080</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -9706,13 +9712,13 @@
     <xdr:from>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>44</xdr:col>
       <xdr:colOff>91440</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>119380</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -9762,13 +9768,13 @@
     <xdr:from>
       <xdr:col>40</xdr:col>
       <xdr:colOff>25400</xdr:colOff>
-      <xdr:row>21</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>101600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>42</xdr:col>
       <xdr:colOff>45720</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:row>23</xdr:row>
       <xdr:rowOff>81280</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -9853,13 +9859,13 @@
     <xdr:from>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2540</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>149860</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>38</xdr:col>
       <xdr:colOff>74930</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>7620</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -9909,14 +9915,14 @@
     <xdr:from>
       <xdr:col>31</xdr:col>
       <xdr:colOff>73660</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>154940</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>40</xdr:col>
-      <xdr:colOff>76200</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>134620</xdr:rowOff>
+      <xdr:col>43</xdr:col>
+      <xdr:colOff>17780</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -9931,8 +9937,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4089400" y="3873500"/>
-          <a:ext cx="1168400" cy="139700"/>
+          <a:off x="4089400" y="3810000"/>
+          <a:ext cx="1498600" cy="279400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -18071,7 +18077,7 @@
   <sheetPr>
     <tabColor rgb="FFFFCCFF"/>
   </sheetPr>
-  <dimension ref="A1:AZ9"/>
+  <dimension ref="A1:AZ10"/>
   <sheetFormatPr defaultColWidth="1.88671875" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="50" width="1.88671875" style="1"/>
@@ -18301,6 +18307,11 @@
     <row r="9" spans="1:52" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C9" s="48" t="s">
         <v>387</v>
+      </c>
+    </row>
+    <row r="10" spans="1:52" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C10" s="48" t="s">
+        <v>388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync(workvault): 2026-10-27 10:12 差分 3 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/LNB管理手順書案_未承認.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/LNB管理手順書案_未承認.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nk365-my.sharepoint.com/personal/ss80751_ad_nkc_co_jp/Documents/ドキュメント/Work_Vault/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="6_{C0F3EAFA-DEEC-4CD0-B5EF-21988F4F198C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1BA0FD4-6038-4310-B888-CC80A25024F8}"/>
+  <xr:revisionPtr revIDLastSave="197" documentId="6_{C0F3EAFA-DEEC-4CD0-B5EF-21988F4F198C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5183834B-EF14-44DC-82D6-9B2B83859BBD}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="表紙" sheetId="18" r:id="rId1"/>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="396">
   <si>
     <t>手 順 書</t>
   </si>
@@ -1463,6 +1463,27 @@
   <si>
     <t>配置：A4縦1頁。事象別の図(アンドン・稼働モニタ異常/月次再起動/異常時再起動)は確実構成図.drawioに残置</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>図1 LNB構成情報画面(出典：LWS 実機画面 2026-10-14 撮影。要確認34の実物。認証IDは伏字)</t>
+  </si>
+  <si>
+    <t>図2 個別スイッチ画面(出典：LWS 実機画面 2026-10-14 撮影。要確認36：192.168.0.1が赤表示)</t>
+  </si>
+  <si>
+    <t>図3 再起動系メニュー(出典：LWS 実機画面 2026-10-14 撮影。要確認30の実物：3ボタンを確認)</t>
+  </si>
+  <si>
+    <t>参考添付：DGS のジョブ設定画面(出典：DGS_P2ジョブ作成シート。LNB のバックアップ手順との対応は未確認)</t>
+  </si>
+  <si>
+    <t>参考添付1 DGS メニュー(データ作成ジョブ一覧)(出典：DGS_P2ジョブ作成シート r007。対応：未確認)</t>
+  </si>
+  <si>
+    <t>参考添付2 DGS データ作成ジョブ一覧(出典：DGS_P2ジョブ作成シート r016。対応：未確認)</t>
+  </si>
+  <si>
+    <t>参考添付3 DGS データ作成ジョブ詳細(出典：DGS_P2ジョブ作成シート r034。対応：未確認)</t>
   </si>
 </sst>
 </file>
@@ -2244,6 +2265,79 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2285,15 +2379,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="3" applyFont="1" applyBorder="1"/>
@@ -2304,70 +2389,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -6479,6 +6500,161 @@
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>53702</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="img_K31">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{66BCEDAD-6EFB-D665-5118-D075943020D2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="259080" y="5501640"/>
+          <a:ext cx="3292202" cy="3810000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>92607</xdr:colOff>
+      <xdr:row>78</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="img_K56">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A715F098-0CA2-7F66-6C41-98698EFB8F30}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="259080" y="9502140"/>
+          <a:ext cx="3460647" cy="3810000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>160019</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>43180</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>96547</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="img_K81">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F4FDB98-A9B5-6637-EBC1-482BD41B7E9C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="259080" y="13502639"/>
+          <a:ext cx="4318000" cy="3136928"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>3</xdr:col>
@@ -10025,6 +10201,161 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="img_B19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA458F2D-48A2-ADCA-AACF-4AAE342BF8D3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="259080" y="3558540"/>
+          <a:ext cx="1314450" cy="1066800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>24765</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>87630</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="img_B27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{31A0A02F-1E56-71ED-7224-0DBC2C7B815A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="259080" y="4838700"/>
+          <a:ext cx="1838325" cy="1847850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="absolute">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>74295</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>102870</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="img_B40">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A7D22B6A-FEBE-92BD-6D22-78CE134C551C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="259080" y="6918960"/>
+          <a:ext cx="4219575" cy="2343150"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -10976,102 +11307,102 @@
       </c>
       <c r="N1" s="25"/>
       <c r="O1" s="26"/>
-      <c r="P1" s="104"/>
-      <c r="Q1" s="105"/>
-      <c r="R1" s="105"/>
-      <c r="S1" s="105"/>
-      <c r="T1" s="105"/>
-      <c r="U1" s="105"/>
-      <c r="V1" s="106"/>
+      <c r="P1" s="76"/>
+      <c r="Q1" s="77"/>
+      <c r="R1" s="77"/>
+      <c r="S1" s="77"/>
+      <c r="T1" s="77"/>
+      <c r="U1" s="77"/>
+      <c r="V1" s="78"/>
       <c r="W1" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="99" t="s">
+      <c r="X1" s="79" t="s">
         <v>347</v>
       </c>
-      <c r="Y1" s="100"/>
+      <c r="Y1" s="80"/>
     </row>
     <row r="2" spans="1:25" ht="58.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="29"/>
       <c r="B2" s="30"/>
-      <c r="D2" s="101" t="s">
+      <c r="D2" s="81" t="s">
         <v>348</v>
       </c>
-      <c r="E2" s="102"/>
-      <c r="F2" s="102"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="102"/>
-      <c r="I2" s="102"/>
-      <c r="J2" s="102"/>
-      <c r="K2" s="102"/>
-      <c r="L2" s="102"/>
-      <c r="M2" s="102"/>
-      <c r="N2" s="102"/>
-      <c r="O2" s="102"/>
-      <c r="P2" s="102"/>
-      <c r="Q2" s="102"/>
-      <c r="R2" s="102"/>
-      <c r="S2" s="102"/>
-      <c r="T2" s="102"/>
-      <c r="U2" s="102"/>
-      <c r="V2" s="102"/>
-      <c r="W2" s="102"/>
+      <c r="E2" s="82"/>
+      <c r="F2" s="82"/>
+      <c r="G2" s="82"/>
+      <c r="H2" s="82"/>
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+      <c r="K2" s="82"/>
+      <c r="L2" s="82"/>
+      <c r="M2" s="82"/>
+      <c r="N2" s="82"/>
+      <c r="O2" s="82"/>
+      <c r="P2" s="82"/>
+      <c r="Q2" s="82"/>
+      <c r="R2" s="82"/>
+      <c r="S2" s="82"/>
+      <c r="T2" s="82"/>
+      <c r="U2" s="82"/>
+      <c r="V2" s="82"/>
+      <c r="W2" s="82"/>
       <c r="X2" s="31"/>
       <c r="Y2" s="23"/>
     </row>
     <row r="3" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="32"/>
       <c r="B3" s="33"/>
-      <c r="D3" s="103" t="s">
+      <c r="D3" s="83" t="s">
         <v>349</v>
       </c>
-      <c r="E3" s="103"/>
-      <c r="F3" s="103"/>
-      <c r="G3" s="103"/>
-      <c r="H3" s="103"/>
-      <c r="I3" s="103"/>
-      <c r="J3" s="103"/>
-      <c r="K3" s="103"/>
-      <c r="L3" s="103"/>
-      <c r="M3" s="103"/>
-      <c r="N3" s="103"/>
-      <c r="O3" s="103"/>
-      <c r="P3" s="103"/>
-      <c r="Q3" s="103"/>
-      <c r="R3" s="103"/>
-      <c r="S3" s="103"/>
-      <c r="T3" s="103"/>
-      <c r="U3" s="103"/>
-      <c r="V3" s="103"/>
-      <c r="W3" s="103"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
+      <c r="J3" s="83"/>
+      <c r="K3" s="83"/>
+      <c r="L3" s="83"/>
+      <c r="M3" s="83"/>
+      <c r="N3" s="83"/>
+      <c r="O3" s="83"/>
+      <c r="P3" s="83"/>
+      <c r="Q3" s="83"/>
+      <c r="R3" s="83"/>
+      <c r="S3" s="83"/>
+      <c r="T3" s="83"/>
+      <c r="U3" s="83"/>
+      <c r="V3" s="83"/>
+      <c r="W3" s="83"/>
       <c r="X3" s="33"/>
       <c r="Y3" s="34"/>
     </row>
     <row r="4" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="32"/>
       <c r="B4" s="33"/>
-      <c r="D4" s="103" t="s">
+      <c r="D4" s="83" t="s">
         <v>350</v>
       </c>
-      <c r="E4" s="103"/>
-      <c r="F4" s="103"/>
-      <c r="G4" s="103"/>
-      <c r="H4" s="103"/>
-      <c r="I4" s="103"/>
-      <c r="J4" s="103"/>
-      <c r="K4" s="103"/>
-      <c r="L4" s="103"/>
-      <c r="M4" s="103"/>
-      <c r="N4" s="103"/>
-      <c r="O4" s="103"/>
-      <c r="P4" s="103"/>
-      <c r="Q4" s="103"/>
-      <c r="R4" s="103"/>
-      <c r="S4" s="103"/>
-      <c r="T4" s="103"/>
-      <c r="U4" s="103"/>
-      <c r="V4" s="103"/>
-      <c r="W4" s="103"/>
+      <c r="E4" s="83"/>
+      <c r="F4" s="83"/>
+      <c r="G4" s="83"/>
+      <c r="H4" s="83"/>
+      <c r="I4" s="83"/>
+      <c r="J4" s="83"/>
+      <c r="K4" s="83"/>
+      <c r="L4" s="83"/>
+      <c r="M4" s="83"/>
+      <c r="N4" s="83"/>
+      <c r="O4" s="83"/>
+      <c r="P4" s="83"/>
+      <c r="Q4" s="83"/>
+      <c r="R4" s="83"/>
+      <c r="S4" s="83"/>
+      <c r="T4" s="83"/>
+      <c r="U4" s="83"/>
+      <c r="V4" s="83"/>
+      <c r="W4" s="83"/>
       <c r="X4" s="33"/>
       <c r="Y4" s="34"/>
     </row>
@@ -11115,21 +11446,21 @@
       <c r="K6" s="33"/>
       <c r="L6" s="36"/>
       <c r="M6" s="36"/>
-      <c r="O6" s="104" t="s">
+      <c r="O6" s="76" t="s">
         <v>351</v>
       </c>
-      <c r="P6" s="105"/>
-      <c r="Q6" s="106"/>
-      <c r="R6" s="104" t="s">
+      <c r="P6" s="77"/>
+      <c r="Q6" s="78"/>
+      <c r="R6" s="76" t="s">
         <v>352</v>
       </c>
-      <c r="S6" s="105"/>
-      <c r="T6" s="106"/>
-      <c r="U6" s="104" t="s">
+      <c r="S6" s="77"/>
+      <c r="T6" s="78"/>
+      <c r="U6" s="76" t="s">
         <v>353</v>
       </c>
-      <c r="V6" s="105"/>
-      <c r="W6" s="106"/>
+      <c r="V6" s="77"/>
+      <c r="W6" s="78"/>
       <c r="Y6" s="34"/>
     </row>
     <row r="7" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -11146,15 +11477,15 @@
       <c r="K7" s="33"/>
       <c r="L7" s="36"/>
       <c r="M7" s="36"/>
-      <c r="O7" s="107"/>
-      <c r="P7" s="108"/>
-      <c r="Q7" s="109"/>
-      <c r="R7" s="107"/>
-      <c r="S7" s="108"/>
-      <c r="T7" s="109"/>
-      <c r="U7" s="107"/>
-      <c r="V7" s="108"/>
-      <c r="W7" s="109"/>
+      <c r="O7" s="67"/>
+      <c r="P7" s="68"/>
+      <c r="Q7" s="69"/>
+      <c r="R7" s="67"/>
+      <c r="S7" s="68"/>
+      <c r="T7" s="69"/>
+      <c r="U7" s="67"/>
+      <c r="V7" s="68"/>
+      <c r="W7" s="69"/>
       <c r="Y7" s="34"/>
     </row>
     <row r="8" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -11171,15 +11502,15 @@
       <c r="K8" s="33"/>
       <c r="L8" s="36"/>
       <c r="M8" s="36"/>
-      <c r="O8" s="110"/>
-      <c r="P8" s="111"/>
-      <c r="Q8" s="112"/>
-      <c r="R8" s="110"/>
-      <c r="S8" s="111"/>
-      <c r="T8" s="112"/>
-      <c r="U8" s="110"/>
-      <c r="V8" s="111"/>
-      <c r="W8" s="112"/>
+      <c r="O8" s="70"/>
+      <c r="P8" s="71"/>
+      <c r="Q8" s="72"/>
+      <c r="R8" s="70"/>
+      <c r="S8" s="71"/>
+      <c r="T8" s="72"/>
+      <c r="U8" s="70"/>
+      <c r="V8" s="71"/>
+      <c r="W8" s="72"/>
       <c r="Y8" s="34"/>
     </row>
     <row r="9" spans="1:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -11223,18 +11554,18 @@
       <c r="L10" s="36"/>
       <c r="M10" s="36"/>
       <c r="N10" s="36"/>
-      <c r="P10" s="113" t="s">
+      <c r="P10" s="73" t="s">
         <v>354</v>
       </c>
-      <c r="Q10" s="113"/>
-      <c r="R10" s="113"/>
-      <c r="S10" s="114" t="s">
+      <c r="Q10" s="73"/>
+      <c r="R10" s="73"/>
+      <c r="S10" s="74" t="s">
         <v>355</v>
       </c>
-      <c r="T10" s="114"/>
-      <c r="U10" s="114"/>
-      <c r="V10" s="114"/>
-      <c r="W10" s="114"/>
+      <c r="T10" s="74"/>
+      <c r="U10" s="74"/>
+      <c r="V10" s="74"/>
+      <c r="W10" s="74"/>
       <c r="Y10" s="34"/>
     </row>
     <row r="11" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -11252,27 +11583,27 @@
       <c r="L11" s="36"/>
       <c r="M11" s="36"/>
       <c r="N11" s="36"/>
-      <c r="P11" s="97" t="s">
+      <c r="P11" s="66" t="s">
         <v>356</v>
       </c>
-      <c r="Q11" s="97"/>
-      <c r="R11" s="97"/>
-      <c r="S11" s="115" t="s">
+      <c r="Q11" s="66"/>
+      <c r="R11" s="66"/>
+      <c r="S11" s="75" t="s">
         <v>355</v>
       </c>
-      <c r="T11" s="115"/>
-      <c r="U11" s="115"/>
-      <c r="V11" s="115"/>
-      <c r="W11" s="115"/>
+      <c r="T11" s="75"/>
+      <c r="U11" s="75"/>
+      <c r="V11" s="75"/>
+      <c r="W11" s="75"/>
       <c r="Y11" s="34"/>
     </row>
     <row r="12" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="37"/>
-      <c r="P12" s="97" t="s">
+      <c r="P12" s="66" t="s">
         <v>357</v>
       </c>
-      <c r="Q12" s="97"/>
-      <c r="R12" s="97"/>
+      <c r="Q12" s="66"/>
+      <c r="R12" s="66"/>
       <c r="S12" s="38"/>
       <c r="T12" s="38"/>
       <c r="U12" s="39" t="s">
@@ -11294,642 +11625,642 @@
         <v>360</v>
       </c>
       <c r="B14" s="44"/>
-      <c r="C14" s="95"/>
-      <c r="D14" s="97"/>
-      <c r="E14" s="97"/>
-      <c r="F14" s="96"/>
-      <c r="G14" s="95"/>
-      <c r="H14" s="97"/>
-      <c r="I14" s="97"/>
-      <c r="J14" s="96"/>
-      <c r="K14" s="98"/>
-      <c r="L14" s="93"/>
-      <c r="M14" s="93"/>
-      <c r="N14" s="93"/>
-      <c r="O14" s="93"/>
-      <c r="P14" s="93"/>
-      <c r="Q14" s="94"/>
-      <c r="R14" s="95"/>
-      <c r="S14" s="96"/>
-      <c r="T14" s="95"/>
-      <c r="U14" s="97"/>
-      <c r="V14" s="97"/>
-      <c r="W14" s="96"/>
-      <c r="X14" s="95"/>
-      <c r="Y14" s="96"/>
+      <c r="C14" s="84"/>
+      <c r="D14" s="66"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="85"/>
+      <c r="G14" s="84"/>
+      <c r="H14" s="66"/>
+      <c r="I14" s="66"/>
+      <c r="J14" s="85"/>
+      <c r="K14" s="86"/>
+      <c r="L14" s="87"/>
+      <c r="M14" s="87"/>
+      <c r="N14" s="87"/>
+      <c r="O14" s="87"/>
+      <c r="P14" s="87"/>
+      <c r="Q14" s="88"/>
+      <c r="R14" s="84"/>
+      <c r="S14" s="85"/>
+      <c r="T14" s="84"/>
+      <c r="U14" s="66"/>
+      <c r="V14" s="66"/>
+      <c r="W14" s="85"/>
+      <c r="X14" s="84"/>
+      <c r="Y14" s="85"/>
     </row>
     <row r="15" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B15" s="44"/>
-      <c r="C15" s="95"/>
-      <c r="D15" s="97"/>
-      <c r="E15" s="97"/>
-      <c r="F15" s="96"/>
-      <c r="G15" s="95"/>
-      <c r="H15" s="97"/>
-      <c r="I15" s="97"/>
-      <c r="J15" s="96"/>
-      <c r="K15" s="98"/>
-      <c r="L15" s="93"/>
-      <c r="M15" s="93"/>
-      <c r="N15" s="93"/>
-      <c r="O15" s="93"/>
-      <c r="P15" s="93"/>
-      <c r="Q15" s="94"/>
-      <c r="R15" s="95"/>
-      <c r="S15" s="96"/>
-      <c r="T15" s="95"/>
-      <c r="U15" s="97"/>
-      <c r="V15" s="97"/>
-      <c r="W15" s="96"/>
-      <c r="X15" s="95"/>
-      <c r="Y15" s="96"/>
+      <c r="C15" s="84"/>
+      <c r="D15" s="66"/>
+      <c r="E15" s="66"/>
+      <c r="F15" s="85"/>
+      <c r="G15" s="84"/>
+      <c r="H15" s="66"/>
+      <c r="I15" s="66"/>
+      <c r="J15" s="85"/>
+      <c r="K15" s="86"/>
+      <c r="L15" s="87"/>
+      <c r="M15" s="87"/>
+      <c r="N15" s="87"/>
+      <c r="O15" s="87"/>
+      <c r="P15" s="87"/>
+      <c r="Q15" s="88"/>
+      <c r="R15" s="84"/>
+      <c r="S15" s="85"/>
+      <c r="T15" s="84"/>
+      <c r="U15" s="66"/>
+      <c r="V15" s="66"/>
+      <c r="W15" s="85"/>
+      <c r="X15" s="84"/>
+      <c r="Y15" s="85"/>
     </row>
     <row r="16" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B16" s="44"/>
-      <c r="C16" s="95"/>
-      <c r="D16" s="97"/>
-      <c r="E16" s="97"/>
-      <c r="F16" s="96"/>
-      <c r="G16" s="95"/>
-      <c r="H16" s="97"/>
-      <c r="I16" s="97"/>
-      <c r="J16" s="96"/>
-      <c r="K16" s="98"/>
-      <c r="L16" s="93"/>
-      <c r="M16" s="93"/>
-      <c r="N16" s="93"/>
-      <c r="O16" s="93"/>
-      <c r="P16" s="93"/>
-      <c r="Q16" s="94"/>
-      <c r="R16" s="95"/>
-      <c r="S16" s="96"/>
-      <c r="T16" s="95"/>
-      <c r="U16" s="97"/>
-      <c r="V16" s="97"/>
-      <c r="W16" s="96"/>
-      <c r="X16" s="95"/>
-      <c r="Y16" s="96"/>
+      <c r="C16" s="84"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="85"/>
+      <c r="G16" s="84"/>
+      <c r="H16" s="66"/>
+      <c r="I16" s="66"/>
+      <c r="J16" s="85"/>
+      <c r="K16" s="86"/>
+      <c r="L16" s="87"/>
+      <c r="M16" s="87"/>
+      <c r="N16" s="87"/>
+      <c r="O16" s="87"/>
+      <c r="P16" s="87"/>
+      <c r="Q16" s="88"/>
+      <c r="R16" s="84"/>
+      <c r="S16" s="85"/>
+      <c r="T16" s="84"/>
+      <c r="U16" s="66"/>
+      <c r="V16" s="66"/>
+      <c r="W16" s="85"/>
+      <c r="X16" s="84"/>
+      <c r="Y16" s="85"/>
     </row>
     <row r="17" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B17" s="44"/>
-      <c r="C17" s="95"/>
-      <c r="D17" s="97"/>
-      <c r="E17" s="97"/>
-      <c r="F17" s="96"/>
-      <c r="G17" s="95"/>
-      <c r="H17" s="97"/>
-      <c r="I17" s="97"/>
-      <c r="J17" s="96"/>
-      <c r="K17" s="98"/>
-      <c r="L17" s="93"/>
-      <c r="M17" s="93"/>
-      <c r="N17" s="93"/>
-      <c r="O17" s="93"/>
-      <c r="P17" s="93"/>
-      <c r="Q17" s="94"/>
-      <c r="R17" s="95"/>
-      <c r="S17" s="96"/>
-      <c r="T17" s="95"/>
-      <c r="U17" s="97"/>
-      <c r="V17" s="97"/>
-      <c r="W17" s="96"/>
-      <c r="X17" s="95"/>
-      <c r="Y17" s="96"/>
+      <c r="C17" s="84"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="66"/>
+      <c r="F17" s="85"/>
+      <c r="G17" s="84"/>
+      <c r="H17" s="66"/>
+      <c r="I17" s="66"/>
+      <c r="J17" s="85"/>
+      <c r="K17" s="86"/>
+      <c r="L17" s="87"/>
+      <c r="M17" s="87"/>
+      <c r="N17" s="87"/>
+      <c r="O17" s="87"/>
+      <c r="P17" s="87"/>
+      <c r="Q17" s="88"/>
+      <c r="R17" s="84"/>
+      <c r="S17" s="85"/>
+      <c r="T17" s="84"/>
+      <c r="U17" s="66"/>
+      <c r="V17" s="66"/>
+      <c r="W17" s="85"/>
+      <c r="X17" s="84"/>
+      <c r="Y17" s="85"/>
     </row>
     <row r="18" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B18" s="44"/>
-      <c r="C18" s="95"/>
-      <c r="D18" s="97"/>
-      <c r="E18" s="97"/>
-      <c r="F18" s="96"/>
-      <c r="G18" s="95"/>
-      <c r="H18" s="97"/>
-      <c r="I18" s="97"/>
-      <c r="J18" s="96"/>
-      <c r="K18" s="98"/>
-      <c r="L18" s="93"/>
-      <c r="M18" s="93"/>
-      <c r="N18" s="93"/>
-      <c r="O18" s="93"/>
-      <c r="P18" s="93"/>
-      <c r="Q18" s="94"/>
-      <c r="R18" s="95"/>
-      <c r="S18" s="96"/>
-      <c r="T18" s="95"/>
-      <c r="U18" s="97"/>
-      <c r="V18" s="97"/>
-      <c r="W18" s="96"/>
-      <c r="X18" s="95"/>
-      <c r="Y18" s="96"/>
+      <c r="C18" s="84"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="85"/>
+      <c r="G18" s="84"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="66"/>
+      <c r="J18" s="85"/>
+      <c r="K18" s="86"/>
+      <c r="L18" s="87"/>
+      <c r="M18" s="87"/>
+      <c r="N18" s="87"/>
+      <c r="O18" s="87"/>
+      <c r="P18" s="87"/>
+      <c r="Q18" s="88"/>
+      <c r="R18" s="84"/>
+      <c r="S18" s="85"/>
+      <c r="T18" s="84"/>
+      <c r="U18" s="66"/>
+      <c r="V18" s="66"/>
+      <c r="W18" s="85"/>
+      <c r="X18" s="84"/>
+      <c r="Y18" s="85"/>
     </row>
     <row r="19" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B19" s="44"/>
-      <c r="C19" s="95"/>
-      <c r="D19" s="97"/>
-      <c r="E19" s="97"/>
-      <c r="F19" s="96"/>
-      <c r="G19" s="95"/>
-      <c r="H19" s="97"/>
-      <c r="I19" s="97"/>
-      <c r="J19" s="96"/>
-      <c r="K19" s="98"/>
-      <c r="L19" s="93"/>
-      <c r="M19" s="93"/>
-      <c r="N19" s="93"/>
-      <c r="O19" s="93"/>
-      <c r="P19" s="93"/>
-      <c r="Q19" s="94"/>
-      <c r="R19" s="95"/>
-      <c r="S19" s="96"/>
-      <c r="T19" s="95"/>
-      <c r="U19" s="97"/>
-      <c r="V19" s="97"/>
-      <c r="W19" s="96"/>
-      <c r="X19" s="95"/>
-      <c r="Y19" s="96"/>
+      <c r="C19" s="84"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="66"/>
+      <c r="F19" s="85"/>
+      <c r="G19" s="84"/>
+      <c r="H19" s="66"/>
+      <c r="I19" s="66"/>
+      <c r="J19" s="85"/>
+      <c r="K19" s="86"/>
+      <c r="L19" s="87"/>
+      <c r="M19" s="87"/>
+      <c r="N19" s="87"/>
+      <c r="O19" s="87"/>
+      <c r="P19" s="87"/>
+      <c r="Q19" s="88"/>
+      <c r="R19" s="84"/>
+      <c r="S19" s="85"/>
+      <c r="T19" s="84"/>
+      <c r="U19" s="66"/>
+      <c r="V19" s="66"/>
+      <c r="W19" s="85"/>
+      <c r="X19" s="84"/>
+      <c r="Y19" s="85"/>
     </row>
     <row r="20" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B20" s="44"/>
-      <c r="C20" s="95"/>
-      <c r="D20" s="97"/>
-      <c r="E20" s="97"/>
-      <c r="F20" s="96"/>
-      <c r="G20" s="95"/>
-      <c r="H20" s="97"/>
-      <c r="I20" s="97"/>
-      <c r="J20" s="96"/>
-      <c r="K20" s="98"/>
-      <c r="L20" s="93"/>
-      <c r="M20" s="93"/>
-      <c r="N20" s="93"/>
-      <c r="O20" s="93"/>
-      <c r="P20" s="93"/>
-      <c r="Q20" s="94"/>
-      <c r="R20" s="95"/>
-      <c r="S20" s="96"/>
-      <c r="T20" s="95"/>
-      <c r="U20" s="97"/>
-      <c r="V20" s="97"/>
-      <c r="W20" s="96"/>
-      <c r="X20" s="95"/>
-      <c r="Y20" s="96"/>
+      <c r="C20" s="84"/>
+      <c r="D20" s="66"/>
+      <c r="E20" s="66"/>
+      <c r="F20" s="85"/>
+      <c r="G20" s="84"/>
+      <c r="H20" s="66"/>
+      <c r="I20" s="66"/>
+      <c r="J20" s="85"/>
+      <c r="K20" s="86"/>
+      <c r="L20" s="87"/>
+      <c r="M20" s="87"/>
+      <c r="N20" s="87"/>
+      <c r="O20" s="87"/>
+      <c r="P20" s="87"/>
+      <c r="Q20" s="88"/>
+      <c r="R20" s="84"/>
+      <c r="S20" s="85"/>
+      <c r="T20" s="84"/>
+      <c r="U20" s="66"/>
+      <c r="V20" s="66"/>
+      <c r="W20" s="85"/>
+      <c r="X20" s="84"/>
+      <c r="Y20" s="85"/>
     </row>
     <row r="21" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B21" s="44"/>
-      <c r="C21" s="95"/>
-      <c r="D21" s="97"/>
-      <c r="E21" s="97"/>
-      <c r="F21" s="96"/>
-      <c r="G21" s="95"/>
-      <c r="H21" s="97"/>
-      <c r="I21" s="97"/>
-      <c r="J21" s="96"/>
-      <c r="K21" s="98"/>
-      <c r="L21" s="93"/>
-      <c r="M21" s="93"/>
-      <c r="N21" s="93"/>
-      <c r="O21" s="93"/>
-      <c r="P21" s="93"/>
-      <c r="Q21" s="94"/>
-      <c r="R21" s="95"/>
-      <c r="S21" s="96"/>
-      <c r="T21" s="95"/>
-      <c r="U21" s="97"/>
-      <c r="V21" s="97"/>
-      <c r="W21" s="96"/>
-      <c r="X21" s="95"/>
-      <c r="Y21" s="96"/>
+      <c r="C21" s="84"/>
+      <c r="D21" s="66"/>
+      <c r="E21" s="66"/>
+      <c r="F21" s="85"/>
+      <c r="G21" s="84"/>
+      <c r="H21" s="66"/>
+      <c r="I21" s="66"/>
+      <c r="J21" s="85"/>
+      <c r="K21" s="86"/>
+      <c r="L21" s="87"/>
+      <c r="M21" s="87"/>
+      <c r="N21" s="87"/>
+      <c r="O21" s="87"/>
+      <c r="P21" s="87"/>
+      <c r="Q21" s="88"/>
+      <c r="R21" s="84"/>
+      <c r="S21" s="85"/>
+      <c r="T21" s="84"/>
+      <c r="U21" s="66"/>
+      <c r="V21" s="66"/>
+      <c r="W21" s="85"/>
+      <c r="X21" s="84"/>
+      <c r="Y21" s="85"/>
     </row>
     <row r="22" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B22" s="44"/>
-      <c r="C22" s="95"/>
-      <c r="D22" s="97"/>
-      <c r="E22" s="97"/>
-      <c r="F22" s="96"/>
-      <c r="G22" s="95"/>
-      <c r="H22" s="97"/>
-      <c r="I22" s="97"/>
-      <c r="J22" s="96"/>
-      <c r="K22" s="98"/>
-      <c r="L22" s="93"/>
-      <c r="M22" s="93"/>
-      <c r="N22" s="93"/>
-      <c r="O22" s="93"/>
-      <c r="P22" s="93"/>
-      <c r="Q22" s="94"/>
-      <c r="R22" s="95"/>
-      <c r="S22" s="96"/>
-      <c r="T22" s="95"/>
-      <c r="U22" s="97"/>
-      <c r="V22" s="97"/>
-      <c r="W22" s="96"/>
-      <c r="X22" s="95"/>
-      <c r="Y22" s="96"/>
+      <c r="C22" s="84"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
+      <c r="F22" s="85"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="66"/>
+      <c r="I22" s="66"/>
+      <c r="J22" s="85"/>
+      <c r="K22" s="86"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="87"/>
+      <c r="N22" s="87"/>
+      <c r="O22" s="87"/>
+      <c r="P22" s="87"/>
+      <c r="Q22" s="88"/>
+      <c r="R22" s="84"/>
+      <c r="S22" s="85"/>
+      <c r="T22" s="84"/>
+      <c r="U22" s="66"/>
+      <c r="V22" s="66"/>
+      <c r="W22" s="85"/>
+      <c r="X22" s="84"/>
+      <c r="Y22" s="85"/>
     </row>
     <row r="23" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B23" s="44"/>
-      <c r="C23" s="95"/>
-      <c r="D23" s="97"/>
-      <c r="E23" s="97"/>
-      <c r="F23" s="96"/>
-      <c r="G23" s="95"/>
-      <c r="H23" s="97"/>
-      <c r="I23" s="97"/>
-      <c r="J23" s="96"/>
-      <c r="K23" s="98"/>
-      <c r="L23" s="93"/>
-      <c r="M23" s="93"/>
-      <c r="N23" s="93"/>
-      <c r="O23" s="93"/>
-      <c r="P23" s="93"/>
-      <c r="Q23" s="94"/>
-      <c r="R23" s="95"/>
-      <c r="S23" s="96"/>
-      <c r="T23" s="95"/>
-      <c r="U23" s="97"/>
-      <c r="V23" s="97"/>
-      <c r="W23" s="96"/>
-      <c r="X23" s="95"/>
-      <c r="Y23" s="96"/>
+      <c r="C23" s="84"/>
+      <c r="D23" s="66"/>
+      <c r="E23" s="66"/>
+      <c r="F23" s="85"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="66"/>
+      <c r="I23" s="66"/>
+      <c r="J23" s="85"/>
+      <c r="K23" s="86"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="87"/>
+      <c r="N23" s="87"/>
+      <c r="O23" s="87"/>
+      <c r="P23" s="87"/>
+      <c r="Q23" s="88"/>
+      <c r="R23" s="84"/>
+      <c r="S23" s="85"/>
+      <c r="T23" s="84"/>
+      <c r="U23" s="66"/>
+      <c r="V23" s="66"/>
+      <c r="W23" s="85"/>
+      <c r="X23" s="84"/>
+      <c r="Y23" s="85"/>
     </row>
     <row r="24" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B24" s="44"/>
-      <c r="C24" s="95"/>
-      <c r="D24" s="97"/>
-      <c r="E24" s="97"/>
-      <c r="F24" s="96"/>
-      <c r="G24" s="95"/>
-      <c r="H24" s="97"/>
-      <c r="I24" s="97"/>
-      <c r="J24" s="96"/>
-      <c r="K24" s="98"/>
-      <c r="L24" s="93"/>
-      <c r="M24" s="93"/>
-      <c r="N24" s="93"/>
-      <c r="O24" s="93"/>
-      <c r="P24" s="93"/>
-      <c r="Q24" s="94"/>
-      <c r="R24" s="95"/>
-      <c r="S24" s="96"/>
-      <c r="T24" s="95"/>
-      <c r="U24" s="97"/>
-      <c r="V24" s="97"/>
-      <c r="W24" s="96"/>
-      <c r="X24" s="95"/>
-      <c r="Y24" s="96"/>
+      <c r="C24" s="84"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
+      <c r="F24" s="85"/>
+      <c r="G24" s="84"/>
+      <c r="H24" s="66"/>
+      <c r="I24" s="66"/>
+      <c r="J24" s="85"/>
+      <c r="K24" s="86"/>
+      <c r="L24" s="87"/>
+      <c r="M24" s="87"/>
+      <c r="N24" s="87"/>
+      <c r="O24" s="87"/>
+      <c r="P24" s="87"/>
+      <c r="Q24" s="88"/>
+      <c r="R24" s="84"/>
+      <c r="S24" s="85"/>
+      <c r="T24" s="84"/>
+      <c r="U24" s="66"/>
+      <c r="V24" s="66"/>
+      <c r="W24" s="85"/>
+      <c r="X24" s="84"/>
+      <c r="Y24" s="85"/>
     </row>
     <row r="25" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B25" s="44"/>
-      <c r="C25" s="95"/>
-      <c r="D25" s="97"/>
-      <c r="E25" s="97"/>
-      <c r="F25" s="96"/>
-      <c r="G25" s="95"/>
-      <c r="H25" s="97"/>
-      <c r="I25" s="97"/>
-      <c r="J25" s="96"/>
-      <c r="K25" s="98"/>
-      <c r="L25" s="93"/>
-      <c r="M25" s="93"/>
-      <c r="N25" s="93"/>
-      <c r="O25" s="93"/>
-      <c r="P25" s="93"/>
-      <c r="Q25" s="94"/>
-      <c r="R25" s="95"/>
-      <c r="S25" s="96"/>
-      <c r="T25" s="95"/>
-      <c r="U25" s="97"/>
-      <c r="V25" s="97"/>
-      <c r="W25" s="96"/>
-      <c r="X25" s="95"/>
-      <c r="Y25" s="96"/>
+      <c r="C25" s="84"/>
+      <c r="D25" s="66"/>
+      <c r="E25" s="66"/>
+      <c r="F25" s="85"/>
+      <c r="G25" s="84"/>
+      <c r="H25" s="66"/>
+      <c r="I25" s="66"/>
+      <c r="J25" s="85"/>
+      <c r="K25" s="86"/>
+      <c r="L25" s="87"/>
+      <c r="M25" s="87"/>
+      <c r="N25" s="87"/>
+      <c r="O25" s="87"/>
+      <c r="P25" s="87"/>
+      <c r="Q25" s="88"/>
+      <c r="R25" s="84"/>
+      <c r="S25" s="85"/>
+      <c r="T25" s="84"/>
+      <c r="U25" s="66"/>
+      <c r="V25" s="66"/>
+      <c r="W25" s="85"/>
+      <c r="X25" s="84"/>
+      <c r="Y25" s="85"/>
     </row>
     <row r="26" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B26" s="44"/>
-      <c r="C26" s="95"/>
-      <c r="D26" s="97"/>
-      <c r="E26" s="97"/>
-      <c r="F26" s="96"/>
-      <c r="G26" s="95"/>
-      <c r="H26" s="97"/>
-      <c r="I26" s="97"/>
-      <c r="J26" s="96"/>
-      <c r="K26" s="98"/>
-      <c r="L26" s="93"/>
-      <c r="M26" s="93"/>
-      <c r="N26" s="93"/>
-      <c r="O26" s="93"/>
-      <c r="P26" s="93"/>
-      <c r="Q26" s="94"/>
-      <c r="R26" s="95"/>
-      <c r="S26" s="96"/>
-      <c r="T26" s="95"/>
-      <c r="U26" s="97"/>
-      <c r="V26" s="97"/>
-      <c r="W26" s="96"/>
-      <c r="X26" s="95"/>
-      <c r="Y26" s="96"/>
+      <c r="C26" s="84"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
+      <c r="F26" s="85"/>
+      <c r="G26" s="84"/>
+      <c r="H26" s="66"/>
+      <c r="I26" s="66"/>
+      <c r="J26" s="85"/>
+      <c r="K26" s="86"/>
+      <c r="L26" s="87"/>
+      <c r="M26" s="87"/>
+      <c r="N26" s="87"/>
+      <c r="O26" s="87"/>
+      <c r="P26" s="87"/>
+      <c r="Q26" s="88"/>
+      <c r="R26" s="84"/>
+      <c r="S26" s="85"/>
+      <c r="T26" s="84"/>
+      <c r="U26" s="66"/>
+      <c r="V26" s="66"/>
+      <c r="W26" s="85"/>
+      <c r="X26" s="84"/>
+      <c r="Y26" s="85"/>
     </row>
     <row r="27" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B27" s="44"/>
-      <c r="C27" s="95"/>
-      <c r="D27" s="97"/>
-      <c r="E27" s="97"/>
-      <c r="F27" s="96"/>
-      <c r="G27" s="95"/>
-      <c r="H27" s="97"/>
-      <c r="I27" s="97"/>
-      <c r="J27" s="96"/>
-      <c r="K27" s="98"/>
-      <c r="L27" s="93"/>
-      <c r="M27" s="93"/>
-      <c r="N27" s="93"/>
-      <c r="O27" s="93"/>
-      <c r="P27" s="93"/>
-      <c r="Q27" s="94"/>
-      <c r="R27" s="95"/>
-      <c r="S27" s="96"/>
-      <c r="T27" s="95"/>
-      <c r="U27" s="97"/>
-      <c r="V27" s="97"/>
-      <c r="W27" s="96"/>
-      <c r="X27" s="95"/>
-      <c r="Y27" s="96"/>
+      <c r="C27" s="84"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
+      <c r="F27" s="85"/>
+      <c r="G27" s="84"/>
+      <c r="H27" s="66"/>
+      <c r="I27" s="66"/>
+      <c r="J27" s="85"/>
+      <c r="K27" s="86"/>
+      <c r="L27" s="87"/>
+      <c r="M27" s="87"/>
+      <c r="N27" s="87"/>
+      <c r="O27" s="87"/>
+      <c r="P27" s="87"/>
+      <c r="Q27" s="88"/>
+      <c r="R27" s="84"/>
+      <c r="S27" s="85"/>
+      <c r="T27" s="84"/>
+      <c r="U27" s="66"/>
+      <c r="V27" s="66"/>
+      <c r="W27" s="85"/>
+      <c r="X27" s="84"/>
+      <c r="Y27" s="85"/>
     </row>
     <row r="28" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B28" s="44"/>
-      <c r="C28" s="95"/>
-      <c r="D28" s="97"/>
-      <c r="E28" s="97"/>
-      <c r="F28" s="96"/>
-      <c r="G28" s="95"/>
-      <c r="H28" s="97"/>
-      <c r="I28" s="97"/>
-      <c r="J28" s="96"/>
-      <c r="K28" s="98"/>
-      <c r="L28" s="93"/>
-      <c r="M28" s="93"/>
-      <c r="N28" s="93"/>
-      <c r="O28" s="93"/>
-      <c r="P28" s="93"/>
-      <c r="Q28" s="94"/>
-      <c r="R28" s="95"/>
-      <c r="S28" s="96"/>
-      <c r="T28" s="95"/>
-      <c r="U28" s="97"/>
-      <c r="V28" s="97"/>
-      <c r="W28" s="96"/>
-      <c r="X28" s="95"/>
-      <c r="Y28" s="96"/>
+      <c r="C28" s="84"/>
+      <c r="D28" s="66"/>
+      <c r="E28" s="66"/>
+      <c r="F28" s="85"/>
+      <c r="G28" s="84"/>
+      <c r="H28" s="66"/>
+      <c r="I28" s="66"/>
+      <c r="J28" s="85"/>
+      <c r="K28" s="86"/>
+      <c r="L28" s="87"/>
+      <c r="M28" s="87"/>
+      <c r="N28" s="87"/>
+      <c r="O28" s="87"/>
+      <c r="P28" s="87"/>
+      <c r="Q28" s="88"/>
+      <c r="R28" s="84"/>
+      <c r="S28" s="85"/>
+      <c r="T28" s="84"/>
+      <c r="U28" s="66"/>
+      <c r="V28" s="66"/>
+      <c r="W28" s="85"/>
+      <c r="X28" s="84"/>
+      <c r="Y28" s="85"/>
     </row>
     <row r="29" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B29" s="44"/>
-      <c r="C29" s="95"/>
-      <c r="D29" s="97"/>
-      <c r="E29" s="97"/>
-      <c r="F29" s="96"/>
-      <c r="G29" s="95"/>
-      <c r="H29" s="97"/>
-      <c r="I29" s="97"/>
-      <c r="J29" s="96"/>
-      <c r="K29" s="98"/>
-      <c r="L29" s="93"/>
-      <c r="M29" s="93"/>
-      <c r="N29" s="93"/>
-      <c r="O29" s="93"/>
-      <c r="P29" s="93"/>
-      <c r="Q29" s="94"/>
-      <c r="R29" s="95"/>
-      <c r="S29" s="96"/>
-      <c r="T29" s="95"/>
-      <c r="U29" s="97"/>
-      <c r="V29" s="97"/>
-      <c r="W29" s="96"/>
-      <c r="X29" s="95"/>
-      <c r="Y29" s="96"/>
+      <c r="C29" s="84"/>
+      <c r="D29" s="66"/>
+      <c r="E29" s="66"/>
+      <c r="F29" s="85"/>
+      <c r="G29" s="84"/>
+      <c r="H29" s="66"/>
+      <c r="I29" s="66"/>
+      <c r="J29" s="85"/>
+      <c r="K29" s="86"/>
+      <c r="L29" s="87"/>
+      <c r="M29" s="87"/>
+      <c r="N29" s="87"/>
+      <c r="O29" s="87"/>
+      <c r="P29" s="87"/>
+      <c r="Q29" s="88"/>
+      <c r="R29" s="84"/>
+      <c r="S29" s="85"/>
+      <c r="T29" s="84"/>
+      <c r="U29" s="66"/>
+      <c r="V29" s="66"/>
+      <c r="W29" s="85"/>
+      <c r="X29" s="84"/>
+      <c r="Y29" s="85"/>
     </row>
     <row r="30" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="43" t="s">
         <v>360</v>
       </c>
       <c r="B30" s="44"/>
-      <c r="C30" s="95"/>
-      <c r="D30" s="97"/>
-      <c r="E30" s="97"/>
-      <c r="F30" s="96"/>
-      <c r="G30" s="95"/>
-      <c r="H30" s="97"/>
-      <c r="I30" s="97"/>
-      <c r="J30" s="96"/>
-      <c r="K30" s="98"/>
-      <c r="L30" s="93"/>
-      <c r="M30" s="93"/>
-      <c r="N30" s="93"/>
-      <c r="O30" s="93"/>
-      <c r="P30" s="93"/>
-      <c r="Q30" s="94"/>
-      <c r="R30" s="95"/>
-      <c r="S30" s="96"/>
-      <c r="T30" s="95"/>
-      <c r="U30" s="97"/>
-      <c r="V30" s="97"/>
-      <c r="W30" s="96"/>
-      <c r="X30" s="95"/>
-      <c r="Y30" s="96"/>
+      <c r="C30" s="84"/>
+      <c r="D30" s="66"/>
+      <c r="E30" s="66"/>
+      <c r="F30" s="85"/>
+      <c r="G30" s="84"/>
+      <c r="H30" s="66"/>
+      <c r="I30" s="66"/>
+      <c r="J30" s="85"/>
+      <c r="K30" s="86"/>
+      <c r="L30" s="87"/>
+      <c r="M30" s="87"/>
+      <c r="N30" s="87"/>
+      <c r="O30" s="87"/>
+      <c r="P30" s="87"/>
+      <c r="Q30" s="88"/>
+      <c r="R30" s="84"/>
+      <c r="S30" s="85"/>
+      <c r="T30" s="84"/>
+      <c r="U30" s="66"/>
+      <c r="V30" s="66"/>
+      <c r="W30" s="85"/>
+      <c r="X30" s="84"/>
+      <c r="Y30" s="85"/>
     </row>
     <row r="31" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="43"/>
       <c r="B31" s="44"/>
-      <c r="C31" s="83"/>
-      <c r="D31" s="84"/>
-      <c r="E31" s="84"/>
-      <c r="F31" s="85"/>
-      <c r="G31" s="83"/>
-      <c r="H31" s="84"/>
-      <c r="I31" s="84"/>
-      <c r="J31" s="85"/>
-      <c r="K31" s="98"/>
-      <c r="L31" s="93"/>
-      <c r="M31" s="93"/>
-      <c r="N31" s="93"/>
-      <c r="O31" s="93"/>
-      <c r="P31" s="93"/>
-      <c r="Q31" s="94"/>
-      <c r="R31" s="95"/>
-      <c r="S31" s="96"/>
-      <c r="T31" s="95"/>
-      <c r="U31" s="97"/>
-      <c r="V31" s="97"/>
-      <c r="W31" s="96"/>
-      <c r="X31" s="95"/>
-      <c r="Y31" s="96"/>
+      <c r="C31" s="89"/>
+      <c r="D31" s="90"/>
+      <c r="E31" s="90"/>
+      <c r="F31" s="91"/>
+      <c r="G31" s="89"/>
+      <c r="H31" s="90"/>
+      <c r="I31" s="90"/>
+      <c r="J31" s="91"/>
+      <c r="K31" s="86"/>
+      <c r="L31" s="87"/>
+      <c r="M31" s="87"/>
+      <c r="N31" s="87"/>
+      <c r="O31" s="87"/>
+      <c r="P31" s="87"/>
+      <c r="Q31" s="88"/>
+      <c r="R31" s="84"/>
+      <c r="S31" s="85"/>
+      <c r="T31" s="84"/>
+      <c r="U31" s="66"/>
+      <c r="V31" s="66"/>
+      <c r="W31" s="85"/>
+      <c r="X31" s="84"/>
+      <c r="Y31" s="85"/>
     </row>
     <row r="32" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="43"/>
       <c r="B32" s="44"/>
-      <c r="C32" s="83"/>
-      <c r="D32" s="84"/>
-      <c r="E32" s="84"/>
-      <c r="F32" s="85"/>
-      <c r="G32" s="83"/>
-      <c r="H32" s="84"/>
-      <c r="I32" s="84"/>
-      <c r="J32" s="85"/>
+      <c r="C32" s="89"/>
+      <c r="D32" s="90"/>
+      <c r="E32" s="90"/>
+      <c r="F32" s="91"/>
+      <c r="G32" s="89"/>
+      <c r="H32" s="90"/>
+      <c r="I32" s="90"/>
+      <c r="J32" s="91"/>
       <c r="K32" s="92"/>
-      <c r="L32" s="93"/>
-      <c r="M32" s="93"/>
-      <c r="N32" s="93"/>
-      <c r="O32" s="93"/>
-      <c r="P32" s="93"/>
-      <c r="Q32" s="94"/>
-      <c r="R32" s="95"/>
-      <c r="S32" s="96"/>
-      <c r="T32" s="95"/>
-      <c r="U32" s="97"/>
-      <c r="V32" s="97"/>
-      <c r="W32" s="96"/>
-      <c r="X32" s="95"/>
-      <c r="Y32" s="96"/>
+      <c r="L32" s="87"/>
+      <c r="M32" s="87"/>
+      <c r="N32" s="87"/>
+      <c r="O32" s="87"/>
+      <c r="P32" s="87"/>
+      <c r="Q32" s="88"/>
+      <c r="R32" s="84"/>
+      <c r="S32" s="85"/>
+      <c r="T32" s="84"/>
+      <c r="U32" s="66"/>
+      <c r="V32" s="66"/>
+      <c r="W32" s="85"/>
+      <c r="X32" s="84"/>
+      <c r="Y32" s="85"/>
     </row>
     <row r="33" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="45"/>
       <c r="B33" s="46"/>
-      <c r="C33" s="83"/>
-      <c r="D33" s="84"/>
-      <c r="E33" s="84"/>
-      <c r="F33" s="85"/>
-      <c r="G33" s="83"/>
-      <c r="H33" s="84"/>
-      <c r="I33" s="84"/>
-      <c r="J33" s="85"/>
-      <c r="K33" s="86"/>
-      <c r="L33" s="87"/>
-      <c r="M33" s="87"/>
-      <c r="N33" s="87"/>
-      <c r="O33" s="87"/>
-      <c r="P33" s="87"/>
-      <c r="Q33" s="88"/>
-      <c r="R33" s="89"/>
-      <c r="S33" s="90"/>
-      <c r="T33" s="89"/>
-      <c r="U33" s="91"/>
-      <c r="V33" s="91"/>
-      <c r="W33" s="90"/>
-      <c r="X33" s="89"/>
-      <c r="Y33" s="90"/>
+      <c r="C33" s="89"/>
+      <c r="D33" s="90"/>
+      <c r="E33" s="90"/>
+      <c r="F33" s="91"/>
+      <c r="G33" s="89"/>
+      <c r="H33" s="90"/>
+      <c r="I33" s="90"/>
+      <c r="J33" s="91"/>
+      <c r="K33" s="110"/>
+      <c r="L33" s="111"/>
+      <c r="M33" s="111"/>
+      <c r="N33" s="111"/>
+      <c r="O33" s="111"/>
+      <c r="P33" s="111"/>
+      <c r="Q33" s="112"/>
+      <c r="R33" s="113"/>
+      <c r="S33" s="114"/>
+      <c r="T33" s="113"/>
+      <c r="U33" s="115"/>
+      <c r="V33" s="115"/>
+      <c r="W33" s="114"/>
+      <c r="X33" s="113"/>
+      <c r="Y33" s="114"/>
     </row>
     <row r="34" spans="1:25" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="66" t="s">
+      <c r="A34" s="93" t="s">
         <v>361</v>
       </c>
-      <c r="B34" s="67"/>
-      <c r="C34" s="70" t="s">
+      <c r="B34" s="94"/>
+      <c r="C34" s="97" t="s">
         <v>362</v>
       </c>
-      <c r="D34" s="71"/>
-      <c r="E34" s="71"/>
-      <c r="F34" s="72"/>
-      <c r="G34" s="70" t="s">
+      <c r="D34" s="98"/>
+      <c r="E34" s="98"/>
+      <c r="F34" s="99"/>
+      <c r="G34" s="97" t="s">
         <v>363</v>
       </c>
-      <c r="H34" s="71"/>
-      <c r="I34" s="71"/>
-      <c r="J34" s="72"/>
-      <c r="K34" s="66" t="s">
+      <c r="H34" s="98"/>
+      <c r="I34" s="98"/>
+      <c r="J34" s="99"/>
+      <c r="K34" s="93" t="s">
         <v>364</v>
       </c>
-      <c r="L34" s="76"/>
-      <c r="M34" s="76"/>
-      <c r="N34" s="76"/>
-      <c r="O34" s="76"/>
-      <c r="P34" s="76"/>
-      <c r="Q34" s="77"/>
-      <c r="R34" s="66" t="s">
+      <c r="L34" s="103"/>
+      <c r="M34" s="103"/>
+      <c r="N34" s="103"/>
+      <c r="O34" s="103"/>
+      <c r="P34" s="103"/>
+      <c r="Q34" s="104"/>
+      <c r="R34" s="93" t="s">
         <v>365</v>
       </c>
-      <c r="S34" s="67"/>
-      <c r="T34" s="66" t="s">
+      <c r="S34" s="94"/>
+      <c r="T34" s="93" t="s">
         <v>366</v>
       </c>
-      <c r="U34" s="81"/>
-      <c r="V34" s="81"/>
-      <c r="W34" s="67"/>
-      <c r="X34" s="66" t="s">
+      <c r="U34" s="108"/>
+      <c r="V34" s="108"/>
+      <c r="W34" s="94"/>
+      <c r="X34" s="93" t="s">
         <v>367</v>
       </c>
-      <c r="Y34" s="67"/>
+      <c r="Y34" s="94"/>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A35" s="68"/>
-      <c r="B35" s="69"/>
-      <c r="C35" s="73"/>
-      <c r="D35" s="74"/>
-      <c r="E35" s="74"/>
-      <c r="F35" s="75"/>
-      <c r="G35" s="73"/>
-      <c r="H35" s="74"/>
-      <c r="I35" s="74"/>
-      <c r="J35" s="75"/>
-      <c r="K35" s="78"/>
-      <c r="L35" s="79"/>
-      <c r="M35" s="79"/>
-      <c r="N35" s="79"/>
-      <c r="O35" s="79"/>
-      <c r="P35" s="79"/>
-      <c r="Q35" s="80"/>
-      <c r="R35" s="68"/>
-      <c r="S35" s="69"/>
-      <c r="T35" s="68"/>
-      <c r="U35" s="82"/>
-      <c r="V35" s="82"/>
-      <c r="W35" s="69"/>
-      <c r="X35" s="68"/>
-      <c r="Y35" s="69"/>
+      <c r="A35" s="95"/>
+      <c r="B35" s="96"/>
+      <c r="C35" s="100"/>
+      <c r="D35" s="101"/>
+      <c r="E35" s="101"/>
+      <c r="F35" s="102"/>
+      <c r="G35" s="100"/>
+      <c r="H35" s="101"/>
+      <c r="I35" s="101"/>
+      <c r="J35" s="102"/>
+      <c r="K35" s="105"/>
+      <c r="L35" s="106"/>
+      <c r="M35" s="106"/>
+      <c r="N35" s="106"/>
+      <c r="O35" s="106"/>
+      <c r="P35" s="106"/>
+      <c r="Q35" s="107"/>
+      <c r="R35" s="95"/>
+      <c r="S35" s="96"/>
+      <c r="T35" s="95"/>
+      <c r="U35" s="109"/>
+      <c r="V35" s="109"/>
+      <c r="W35" s="96"/>
+      <c r="X35" s="95"/>
+      <c r="Y35" s="96"/>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A36" s="47" t="s">
@@ -11944,15 +12275,116 @@
     </row>
   </sheetData>
   <mergeCells count="143">
-    <mergeCell ref="P12:R12"/>
-    <mergeCell ref="O7:Q8"/>
-    <mergeCell ref="R7:T8"/>
-    <mergeCell ref="U7:W8"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="S10:W10"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="S11:W11"/>
-    <mergeCell ref="P1:V1"/>
+    <mergeCell ref="X34:Y35"/>
+    <mergeCell ref="A34:B35"/>
+    <mergeCell ref="C34:F35"/>
+    <mergeCell ref="G34:J35"/>
+    <mergeCell ref="K34:Q35"/>
+    <mergeCell ref="R34:S35"/>
+    <mergeCell ref="T34:W35"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="K33:Q33"/>
+    <mergeCell ref="R33:S33"/>
+    <mergeCell ref="T33:W33"/>
+    <mergeCell ref="X33:Y33"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="K32:Q32"/>
+    <mergeCell ref="R32:S32"/>
+    <mergeCell ref="T32:W32"/>
+    <mergeCell ref="X32:Y32"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K31:Q31"/>
+    <mergeCell ref="R31:S31"/>
+    <mergeCell ref="T31:W31"/>
+    <mergeCell ref="X31:Y31"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="K30:Q30"/>
+    <mergeCell ref="R30:S30"/>
+    <mergeCell ref="T30:W30"/>
+    <mergeCell ref="X30:Y30"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="K29:Q29"/>
+    <mergeCell ref="R29:S29"/>
+    <mergeCell ref="T29:W29"/>
+    <mergeCell ref="X29:Y29"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="K28:Q28"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="T28:W28"/>
+    <mergeCell ref="X28:Y28"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="K27:Q27"/>
+    <mergeCell ref="R27:S27"/>
+    <mergeCell ref="T27:W27"/>
+    <mergeCell ref="X27:Y27"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="K26:Q26"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="T26:W26"/>
+    <mergeCell ref="X26:Y26"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="K25:Q25"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="T25:W25"/>
+    <mergeCell ref="X25:Y25"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K24:Q24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="T24:W24"/>
+    <mergeCell ref="X24:Y24"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="K23:Q23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="T23:W23"/>
+    <mergeCell ref="X23:Y23"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="K22:Q22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="T22:W22"/>
+    <mergeCell ref="X22:Y22"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K21:Q21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="T21:W21"/>
+    <mergeCell ref="X21:Y21"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="K20:Q20"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="T20:W20"/>
+    <mergeCell ref="X20:Y20"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="K19:Q19"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="T19:W19"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="T14:W14"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="K18:Q18"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="T18:W18"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="K17:Q17"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="T17:W17"/>
+    <mergeCell ref="X17:Y17"/>
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="D2:W2"/>
     <mergeCell ref="D3:W3"/>
@@ -11977,116 +12409,15 @@
     <mergeCell ref="G14:J14"/>
     <mergeCell ref="K14:Q14"/>
     <mergeCell ref="R14:S14"/>
-    <mergeCell ref="T14:W14"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="K18:Q18"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="T18:W18"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="K17:Q17"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="T17:W17"/>
-    <mergeCell ref="X17:Y17"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="K20:Q20"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="T20:W20"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="K19:Q19"/>
-    <mergeCell ref="R19:S19"/>
-    <mergeCell ref="T19:W19"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="G22:J22"/>
-    <mergeCell ref="K22:Q22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="T22:W22"/>
-    <mergeCell ref="X22:Y22"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K21:Q21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="T21:W21"/>
-    <mergeCell ref="X21:Y21"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K24:Q24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="T24:W24"/>
-    <mergeCell ref="X24:Y24"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="K23:Q23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="T23:W23"/>
-    <mergeCell ref="X23:Y23"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="K26:Q26"/>
-    <mergeCell ref="R26:S26"/>
-    <mergeCell ref="T26:W26"/>
-    <mergeCell ref="X26:Y26"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="K25:Q25"/>
-    <mergeCell ref="R25:S25"/>
-    <mergeCell ref="T25:W25"/>
-    <mergeCell ref="X25:Y25"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="K28:Q28"/>
-    <mergeCell ref="R28:S28"/>
-    <mergeCell ref="T28:W28"/>
-    <mergeCell ref="X28:Y28"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="K27:Q27"/>
-    <mergeCell ref="R27:S27"/>
-    <mergeCell ref="T27:W27"/>
-    <mergeCell ref="X27:Y27"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="K30:Q30"/>
-    <mergeCell ref="R30:S30"/>
-    <mergeCell ref="T30:W30"/>
-    <mergeCell ref="X30:Y30"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="K29:Q29"/>
-    <mergeCell ref="R29:S29"/>
-    <mergeCell ref="T29:W29"/>
-    <mergeCell ref="X29:Y29"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="K32:Q32"/>
-    <mergeCell ref="R32:S32"/>
-    <mergeCell ref="T32:W32"/>
-    <mergeCell ref="X32:Y32"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K31:Q31"/>
-    <mergeCell ref="R31:S31"/>
-    <mergeCell ref="T31:W31"/>
-    <mergeCell ref="X31:Y31"/>
-    <mergeCell ref="X34:Y35"/>
-    <mergeCell ref="A34:B35"/>
-    <mergeCell ref="C34:F35"/>
-    <mergeCell ref="G34:J35"/>
-    <mergeCell ref="K34:Q35"/>
-    <mergeCell ref="R34:S35"/>
-    <mergeCell ref="T34:W35"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="K33:Q33"/>
-    <mergeCell ref="R33:S33"/>
-    <mergeCell ref="T33:W33"/>
-    <mergeCell ref="X33:Y33"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="O7:Q8"/>
+    <mergeCell ref="R7:T8"/>
+    <mergeCell ref="U7:W8"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="S10:W10"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="S11:W11"/>
+    <mergeCell ref="P1:V1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.86614173228346458" right="0.51181102362204722" top="0.59055118110236227" bottom="0.19685039370078741" header="0.59055118110236227" footer="0.19685039370078741"/>
@@ -17678,7 +18009,7 @@
   <sheetPr>
     <tabColor rgb="FFFFCCFF"/>
   </sheetPr>
-  <dimension ref="A1:AZ36"/>
+  <dimension ref="A1:AZ107"/>
   <sheetFormatPr defaultColWidth="1.88671875" defaultRowHeight="12.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="50" width="1.88671875" style="1"/>
@@ -18021,29 +18352,248 @@
         <v>59</v>
       </c>
     </row>
+    <row r="31" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C31" s="13"/>
+    </row>
     <row r="32" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="16" t="s">
+      <c r="C32" s="13"/>
+    </row>
+    <row r="33" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C33" s="13"/>
+    </row>
+    <row r="34" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C34" s="13"/>
+    </row>
+    <row r="35" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C35" s="13"/>
+    </row>
+    <row r="36" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C36" s="13"/>
+    </row>
+    <row r="37" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C37" s="13"/>
+    </row>
+    <row r="38" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C38" s="13"/>
+    </row>
+    <row r="39" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C39" s="13"/>
+    </row>
+    <row r="40" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C40" s="13"/>
+    </row>
+    <row r="41" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C41" s="13"/>
+    </row>
+    <row r="42" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C42" s="13"/>
+    </row>
+    <row r="43" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C43" s="13"/>
+    </row>
+    <row r="44" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C44" s="13"/>
+    </row>
+    <row r="45" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C45" s="13"/>
+    </row>
+    <row r="46" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C46" s="13"/>
+    </row>
+    <row r="47" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C47" s="13"/>
+    </row>
+    <row r="48" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C48" s="13"/>
+    </row>
+    <row r="49" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C49" s="13"/>
+    </row>
+    <row r="50" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C50" s="13"/>
+    </row>
+    <row r="51" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C51" s="13"/>
+    </row>
+    <row r="52" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C52" s="13"/>
+    </row>
+    <row r="53" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C53" s="13"/>
+    </row>
+    <row r="54" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C54" s="13"/>
+    </row>
+    <row r="55" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C55" s="13" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="56" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C56" s="13"/>
+    </row>
+    <row r="57" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C57" s="13"/>
+    </row>
+    <row r="58" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C58" s="13"/>
+    </row>
+    <row r="59" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C59" s="13"/>
+    </row>
+    <row r="60" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C60" s="13"/>
+    </row>
+    <row r="61" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C61" s="13"/>
+    </row>
+    <row r="62" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C62" s="13"/>
+    </row>
+    <row r="63" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C63" s="13"/>
+    </row>
+    <row r="64" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C64" s="13"/>
+    </row>
+    <row r="65" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C65" s="13"/>
+    </row>
+    <row r="66" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C66" s="13"/>
+    </row>
+    <row r="67" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C67" s="13"/>
+    </row>
+    <row r="68" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C68" s="13"/>
+    </row>
+    <row r="69" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C69" s="13"/>
+    </row>
+    <row r="70" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C70" s="13"/>
+    </row>
+    <row r="71" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C71" s="13"/>
+    </row>
+    <row r="72" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C72" s="13"/>
+    </row>
+    <row r="73" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C73" s="13"/>
+    </row>
+    <row r="74" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C74" s="13"/>
+    </row>
+    <row r="75" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C75" s="13"/>
+    </row>
+    <row r="76" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C76" s="13"/>
+    </row>
+    <row r="77" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C77" s="13"/>
+    </row>
+    <row r="78" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C78" s="13"/>
+    </row>
+    <row r="79" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C79" s="13"/>
+    </row>
+    <row r="80" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C80" s="13" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="81" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C81" s="13"/>
+    </row>
+    <row r="82" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C82" s="13"/>
+    </row>
+    <row r="83" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C83" s="13"/>
+    </row>
+    <row r="84" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C84" s="13"/>
+    </row>
+    <row r="85" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C85" s="13"/>
+    </row>
+    <row r="86" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C86" s="13"/>
+    </row>
+    <row r="87" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C87" s="13"/>
+    </row>
+    <row r="88" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C88" s="13"/>
+    </row>
+    <row r="89" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C89" s="13"/>
+    </row>
+    <row r="90" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C90" s="13"/>
+    </row>
+    <row r="91" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C91" s="13"/>
+    </row>
+    <row r="92" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C92" s="13"/>
+    </row>
+    <row r="93" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C93" s="13"/>
+    </row>
+    <row r="94" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C94" s="13"/>
+    </row>
+    <row r="95" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C95" s="13"/>
+    </row>
+    <row r="96" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C96" s="13"/>
+    </row>
+    <row r="97" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C97" s="13"/>
+    </row>
+    <row r="98" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C98" s="13"/>
+    </row>
+    <row r="99" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C99" s="13"/>
+    </row>
+    <row r="100" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C100" s="13"/>
+    </row>
+    <row r="101" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C101" s="13" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="16" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C33" s="13" t="s">
+    <row r="104" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C104" s="13" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C34" s="13" t="s">
+    <row r="105" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C105" s="13" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="C35" s="1" t="s">
+    <row r="106" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C106" s="1" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="17"/>
-      <c r="C36" s="1" t="s">
+    <row r="107" spans="1:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A107" s="17"/>
+      <c r="C107" s="1" t="s">
         <v>383</v>
       </c>
     </row>
@@ -18063,12 +18613,18 @@
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.86614173228346458" right="0.51181102362204722" top="0.59055118110236227" bottom="0.78740157480314965" header="0.59055118110236227" footer="0.39370078740157483"/>
-  <pageSetup paperSize="9" firstPageNumber="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <pageSetup paperSize="9" firstPageNumber="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader>&amp;R
 &amp;P</oddHeader>
     <oddFooter>&amp;L&amp;"ＭＳ ゴシック,標準"　　　NR4030&amp;C&amp;"ＭＳ ゴシック,標準"様式 NR4030-0300-A3&amp;R&amp;"ＭＳ ゴシック,標準"日本光電</oddFooter>
   </headerFooter>
+  <rowBreaks count="3" manualBreakCount="3">
+    <brk id="30" max="16383" man="1"/>
+    <brk id="55" max="16383" man="1"/>
+    <brk id="80" max="16383" man="1"/>
+  </rowBreaks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -19705,7 +20261,27 @@
         <v>113</v>
       </c>
     </row>
-    <row r="59" ht="14.4" x14ac:dyDescent="0.15"/>
+    <row r="18" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C18" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="26" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C26" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="39" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C39" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="55" spans="3:3" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="C55" s="1" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="59" spans="3:3" ht="14.4" x14ac:dyDescent="0.15"/>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="AC3:AZ3"/>
@@ -19722,12 +20298,18 @@
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.86614173228346458" right="0.51181102362204722" top="0.59055118110236227" bottom="0.78740157480314965" header="0.59055118110236227" footer="0.39370078740157483"/>
-  <pageSetup paperSize="9" firstPageNumber="15" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
+  <pageSetup paperSize="9" firstPageNumber="15" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <headerFooter alignWithMargins="0">
     <oddHeader>&amp;R
 &amp;P</oddHeader>
     <oddFooter>&amp;L&amp;"ＭＳ ゴシック,標準"　　　NR4030&amp;C&amp;"ＭＳ ゴシック,標準"様式 NR4030-0300-A3&amp;R&amp;"ＭＳ ゴシック,標準"日本光電</oddFooter>
   </headerFooter>
+  <rowBreaks count="3" manualBreakCount="3">
+    <brk id="18" max="16383" man="1"/>
+    <brk id="26" max="16383" man="1"/>
+    <brk id="39" max="16383" man="1"/>
+  </rowBreaks>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>